<commit_message>
feat: materialize dual respondent evidence architecture
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Dual_Respondent_Axis_Comparison_v1.xlsx
+++ b/NewLogic 03.05.2026/ST_Dual_Respondent_Axis_Comparison_v1.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -135,6 +135,7 @@
       <color rgb="FF1A1A1A"/>
       <sz val="10"/>
     </font>
+    <font/>
   </fonts>
   <fills count="11">
     <fill>
@@ -194,7 +195,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -275,6 +276,7 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -286,7 +288,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -407,6 +409,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -968,7 +980,7 @@
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>Canonical Role × Question legitimate-observation-scope structure and seniority-tier mapping. MATRIX STRUCTURE ONLY — SEPARATE AUTHORING REQUIRED. No production roleCoverageMultiplier until row content is authored.</t>
+          <t>Observation Scope rules layer (Seniority mapping + Question_Tier_Vantage + header-only Role_Question_Override + question-qualified E/F + semantic-class effects + actual-access ceilings). MATERIALIZED METHODOLOGY / GENERATED CORPUS; NOT PRODUCTION-ACTIVE (X-3 S-1/S-2). No roleCoverageMultiplier.</t>
         </is>
       </c>
       <c r="C22" s="26" t="inlineStr">
@@ -978,7 +990,7 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>Seniority tier mapping; empty Role × Question matrix schema</t>
+          <t>Rules layer; seniority mapping; zero Role_Question_Override data rows</t>
         </is>
       </c>
     </row>
@@ -990,7 +1002,7 @@
       </c>
       <c r="B23" s="26" t="inlineStr">
         <is>
-          <t>Sole canonical authority for state-machine evaluation order. Precondition/coverage outcomes are outside the five-state enum.</t>
+          <t>Sole canonical authority for state-machine evaluation order, including 0c UNRESOLVED and 3a one-HIGH DEC-7. Precondition/coverage/routing outcomes are outside the five-state enum.</t>
         </is>
       </c>
       <c r="C23" s="26" t="inlineStr">
@@ -1026,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="14" min="1" max="1"/>
@@ -1392,7 +1404,7 @@
       </c>
       <c r="C19" s="34" t="inlineStr">
         <is>
-          <t>Quality multiplier values (0.3, 0.5, 0.6, 0.7) require independent professional audit per project documented requirement.</t>
+          <t>Quality multiplier values (0.3, 0.5, 0.6, 0.7) require independent professional audit per project documented requirement. D0_R1: mandate remains OPEN and now also includes justification of four-factor multiplication, factor dependencies, Schema vs Dual numeric regime, confidence, reliability flags, thresholds, range, pair-combination rule, empirical calibration, and the DEC-8 ≥ 0.5 PRIMARY × CONTEXTUAL quality gate. No numeric value was changed in D0_R1. Range 0.027 to 1.0 is SUPERSEDED / ANNULLED with no replacement.</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
@@ -1409,7 +1421,7 @@
       </c>
       <c r="B20" s="34" t="inlineStr">
         <is>
-          <t>PENDING — matrix structure defined, row content requires separate methodology authoring act</t>
+          <t>PENDING — methodology/generated corpus materialized as compact rules layer; PRODUCTION-ACTIVE Observation Scope blocked by X-3 S-1/S-2. Row content of a 396-cell numeric matrix is not used. No roleCoverageMultiplier.</t>
         </is>
       </c>
       <c r="C20" s="34" t="inlineStr">
@@ -1420,6 +1432,28 @@
       <c r="D20" s="34" t="inlineStr">
         <is>
           <t>Authoring act required before evidence-quality dimension 5 may be production-computed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Question-qualified E/F semantics and X-2</t>
+        </is>
+      </c>
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>PARTIAL — table materialized; X-2 / Q10 E = AMBIGUOUS_COLLAPSE not repaired</t>
+        </is>
+      </c>
+      <c r="C21" s="34" t="inlineStr">
+        <is>
+          <t>Sheet 11 Block C1: 15 rows. Q11 E = SUBSTANTIVE_SIGNAL. Q8/Q9/Q6 E vs F distinct. No global E/F rule.</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="inlineStr">
+        <is>
+          <t>Do not close X-2 in this workbook. Canonical Schema unchanged.</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="14" min="1" max="1"/>
@@ -1790,6 +1824,28 @@
       <c r="D18" s="32" t="inlineStr">
         <is>
           <t>DR-A / DR-B / DR-C / DR-D + C-21/C-22/C-23/C-24 materialization. Role × Question matrix row content is NOT complete; MATRIX STRUCTURE ONLY — SEPARATE AUTHORING REQUIRED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>15. Owner evidence-architecture pass D0_R1</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>CORRECTED</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>sheets 2 (note only), 3 G5/G7/G9, 4, 5, 7, 8, 9, 10, 11, 12</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>DEC-1…DEC-8, DEC-7b, X-9, question-qualified E/F, Observation Scope rules layer. Supersedes, does not retract, prior role-coverage multiplier language. 0.027 range SUPERSEDED / ANNULLED — no replacement pending C-25/X-4. Four-factor product remains PROVISIONAL. C-25/X-4 OPEN. X-3 OPEN (S-1/S-2 block production-active Observation Scope). X-8 calibration/schema work remains pending. X-9b UI debt remains open (ST_Step3_Output_Screens_Spec.xlsx / reporting.json not edited). X-10 closure; X-11 closure (Owner-accepted). X-1 / X-2 / X-2b / X-3 not repaired. No empirical validation claimed. No runtime implementation.</t>
         </is>
       </c>
     </row>
@@ -1810,37 +1866,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="15" min="1" max="1"/>
-    <col width="36" customWidth="1" style="15" min="2" max="2"/>
-    <col width="70" customWidth="1" style="15" min="3" max="3"/>
-    <col width="42" customWidth="1" style="15" min="4" max="4"/>
-    <col width="28" customWidth="1" style="15" min="5" max="5"/>
-    <col width="36" customWidth="1" style="15" min="6" max="6"/>
+    <col width="16" customWidth="1" style="15" min="1" max="1"/>
+    <col width="18" customWidth="1" style="15" min="2" max="2"/>
+    <col width="42" customWidth="1" style="15" min="3" max="3"/>
+    <col width="28" customWidth="1" style="15" min="4" max="4"/>
+    <col width="22" customWidth="1" style="15" min="5" max="5"/>
+    <col width="42" customWidth="1" style="15" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="15">
-      <c r="A1" s="35" t="inlineStr">
-        <is>
-          <t>ROLE × QUESTION LEGITIMATE OBSERVATION SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" s="15">
-      <c r="A2" s="36" t="inlineStr">
-        <is>
-          <t>STATUS: MATRIX STRUCTURE ONLY — SEPARATE AUTHORING REQUIRED</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1" s="15">
-      <c r="A3" s="36" t="inlineStr">
-        <is>
-          <t>The matrix schema is canonical, but row content has NOT been authored or accepted. No production roleCoverageMultiplier may be computed from an empty matrix. No default, fallback, or 1.0 substitution is permitted.</t>
-        </is>
-      </c>
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>OBSERVATION SCOPE RULES LAYER · sheet 11 · D0_R1</t>
+        </is>
+      </c>
+      <c r="G1" s="43" t="n"/>
+      <c r="H1" s="43" t="n"/>
+    </row>
+    <row r="2" ht="48" customHeight="1" s="15">
+      <c r="A2" s="44" t="inlineStr">
+        <is>
+          <t>STATUS: MATERIALIZED METHODOLOGY / GENERATED CORPUS. NOT PRODUCTION-ACTIVE OBSERVATION SCOPE — blocked by X-3 S-1/S-2. No roleCoverageMultiplier. Seniority is not an evidence-quality score. Application order: C1 → C2 → C3.</t>
+        </is>
+      </c>
+      <c r="G2" s="43" t="n"/>
+      <c r="H2" s="43" t="n"/>
+    </row>
+    <row r="3" ht="56" customHeight="1" s="15">
+      <c r="A3" s="44" t="inlineStr">
+        <is>
+          <t>Use classes (exactly four): PRIMARY · CONTEXTUAL · INELIGIBLE · UNRESOLVED. Chain: enrolment / expected vantage → independent capture → question-specific actual access → Observation Use Class → provisional evidence quality → comparison → divergence diagnosis → bounded corroboration / re-probe → five-state classifier → Contradiction / routing. Final Environment label is not produced.</t>
+        </is>
+      </c>
+      <c r="G3" s="43" t="n"/>
+      <c r="H3" s="43" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="37" t="inlineStr">
@@ -1851,8 +1913,12 @@
       <c r="B4" s="40" t="n"/>
       <c r="C4" s="40" t="n"/>
       <c r="D4" s="41" t="n"/>
-    </row>
-    <row r="5">
+      <c r="E4" s="43" t="n"/>
+      <c r="F4" s="43" t="n"/>
+      <c r="G4" s="43" t="n"/>
+      <c r="H4" s="43" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="15">
       <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Seniority Tier</t>
@@ -1873,8 +1939,12 @@
           <t>Source</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="48" customHeight="1" s="15">
+      <c r="E5" s="43" t="n"/>
+      <c r="F5" s="43" t="n"/>
+      <c r="G5" s="43" t="n"/>
+      <c r="H5" s="43" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1" s="15">
       <c r="A6" s="39" t="inlineStr">
         <is>
           <t>senior</t>
@@ -1895,8 +1965,12 @@
           <t>DR-B2; ST_Canonical_Schema.xlsx v1.1 8_Respondent_Record</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="48" customHeight="1" s="15">
+      <c r="E6" s="43" t="n"/>
+      <c r="F6" s="43" t="n"/>
+      <c r="G6" s="43" t="n"/>
+      <c r="H6" s="43" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1" s="15">
       <c r="A7" s="39" t="inlineStr">
         <is>
           <t>line_level</t>
@@ -1917,8 +1991,12 @@
           <t>DR-B2; Dual Respondent canonical role-level split rules</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="48" customHeight="1" s="15">
+      <c r="E7" s="43" t="n"/>
+      <c r="F7" s="43" t="n"/>
+      <c r="G7" s="43" t="n"/>
+      <c r="H7" s="43" t="n"/>
+    </row>
+    <row r="8" ht="32" customHeight="1" s="15">
       <c r="A8" s="39" t="inlineStr">
         <is>
           <t>external</t>
@@ -1939,66 +2017,1763 @@
           <t>DR-B2</t>
         </is>
       </c>
+      <c r="E8" s="43" t="n"/>
+      <c r="F8" s="43" t="n"/>
+      <c r="G8" s="43" t="n"/>
+      <c r="H8" s="43" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="43" t="n"/>
+      <c r="B9" s="43" t="n"/>
+      <c r="C9" s="43" t="n"/>
+      <c r="D9" s="43" t="n"/>
+      <c r="E9" s="43" t="n"/>
+      <c r="F9" s="43" t="n"/>
+      <c r="G9" s="43" t="n"/>
+      <c r="H9" s="43" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="37" t="inlineStr">
         <is>
-          <t>Role_Question_Observation_Scope</t>
+          <t>BLOCK A — Question_Tier_Vantage</t>
         </is>
       </c>
       <c r="B10" s="40" t="n"/>
       <c r="C10" s="40" t="n"/>
       <c r="D10" s="40" t="n"/>
-      <c r="E10" s="40" t="n"/>
-      <c r="F10" s="41" t="n"/>
-    </row>
-    <row r="11">
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="43" t="n"/>
+      <c r="G10" s="43" t="n"/>
+      <c r="H10" s="43" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1" s="15">
       <c r="A11" s="38" t="inlineStr">
         <is>
+          <t>questionRef</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>seniorityTier</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>expectedVantage</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>defaultUseClass</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>sourceBasis</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="n"/>
+      <c r="G11" s="43" t="n"/>
+      <c r="H11" s="43" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1" s="15">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D12" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+      <c r="F12" s="43" t="n"/>
+      <c r="G12" s="43" t="n"/>
+      <c r="H12" s="43" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="15">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B13" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="inlineStr">
+        <is>
+          <t>CONTEXTUAL</t>
+        </is>
+      </c>
+      <c r="E13" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+      <c r="F13" s="43" t="n"/>
+      <c r="G13" s="43" t="n"/>
+      <c r="H13" s="43" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1" s="15">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" s="15">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D15" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E15" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" s="15">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="inlineStr">
+        <is>
+          <t>INELIGIBLE</t>
+        </is>
+      </c>
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="15">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B17" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D17" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E17" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" s="15">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B18" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D18" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E18" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" s="15">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B19" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D19" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E19" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" s="15">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B20" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D20" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E20" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" s="15">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" s="15">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E22" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" s="15">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" s="15">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D24" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E24" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="15">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>CONTEXTUAL</t>
+        </is>
+      </c>
+      <c r="E25" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" s="15">
+      <c r="A26" s="39" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B26" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D26" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E26" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" s="15">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B27" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C27" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D27" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E27" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" s="15">
+      <c r="A28" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B28" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C28" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D28" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E28" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="15">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B29" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D29" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E29" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" s="15">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B30" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D30" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E30" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" s="15">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B31" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D31" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E31" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" s="15">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B32" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D32" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E32" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="15">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B33" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D33" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E33" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" s="15">
+      <c r="A34" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B34" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C34" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D34" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E34" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" s="15">
+      <c r="A35" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C35" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D35" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E35" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1" s="15">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D36" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1" s="15">
+      <c r="A37" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B37" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C37" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D37" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E37" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1" s="15">
+      <c r="A38" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B38" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D38" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E38" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1" s="15">
+      <c r="A39" s="39" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B39" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E39" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1" s="15">
+      <c r="A40" s="39" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B40" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C40" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D40" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E40" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1" s="15">
+      <c r="A41" s="39" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B41" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C41" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E41" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1" s="15">
+      <c r="A42" s="39" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B42" s="39" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
+      <c r="C42" s="39" t="inlineStr">
+        <is>
+          <t>Governance / decision-authority altitude</t>
+        </is>
+      </c>
+      <c r="D42" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E42" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1" s="15">
+      <c r="A43" s="39" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B43" s="39" t="inlineStr">
+        <is>
+          <t>line_level</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
+        <is>
+          <t>Operational altitude</t>
+        </is>
+      </c>
+      <c r="D43" s="39" t="inlineStr">
+        <is>
+          <t>PRIMARY</t>
+        </is>
+      </c>
+      <c r="E43" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1" s="15">
+      <c r="A44" s="39" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B44" s="39" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="C44" s="39" t="inlineStr">
+        <is>
+          <t>Outside internal seniority ladder</t>
+        </is>
+      </c>
+      <c r="D44" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="E44" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>BLOCK B — Role_Question_Override (header only; no speculative rows)</t>
+        </is>
+      </c>
+      <c r="B46" s="40" t="n"/>
+      <c r="C46" s="40" t="n"/>
+      <c r="D46" s="40" t="n"/>
+      <c r="E46" s="41" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1" s="15">
+      <c r="A47" s="38" t="inlineStr">
+        <is>
           <t>roleCode</t>
         </is>
       </c>
-      <c r="B11" s="38" t="inlineStr">
-        <is>
-          <t>seniorityTier</t>
-        </is>
-      </c>
-      <c r="C11" s="38" t="inlineStr">
+      <c r="B47" s="38" t="inlineStr">
         <is>
           <t>questionRef</t>
         </is>
       </c>
-      <c r="D11" s="38" t="inlineStr">
-        <is>
-          <t>scopeLevel</t>
-        </is>
-      </c>
-      <c r="E11" s="38" t="inlineStr">
-        <is>
-          <t>roleCoverageMultiplier</t>
-        </is>
-      </c>
-      <c r="F11" s="38" t="inlineStr">
+      <c r="C47" s="38" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>useClassCap</t>
+        </is>
+      </c>
+      <c r="E47" s="38" t="inlineStr">
         <is>
           <t>sourceBasis</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1" s="15">
-      <c r="A13" s="36" t="inlineStr">
-        <is>
-          <t>Allowed future enums (prose only; no data rows): seniorityTier = senior / line_level / external / any; questionRef = Q1 … Q11; scopeLevel = full / partial / out_of_scope. DATA ROWS: ZERO. Do not compute a production roleCoverageMultiplier from this empty matrix.</t>
+    <row r="49">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>BLOCK C1 — Question_Option_Semantics</t>
+        </is>
+      </c>
+      <c r="B49" s="40" t="n"/>
+      <c r="C49" s="40" t="n"/>
+      <c r="D49" s="41" t="n"/>
+    </row>
+    <row r="50" ht="22" customHeight="1" s="15">
+      <c r="A50" s="38" t="inlineStr">
+        <is>
+          <t>questionRef</t>
+        </is>
+      </c>
+      <c r="B50" s="38" t="inlineStr">
+        <is>
+          <t>optionCode</t>
+        </is>
+      </c>
+      <c r="C50" s="38" t="inlineStr">
+        <is>
+          <t>semanticClass</t>
+        </is>
+      </c>
+      <c r="D50" s="38" t="inlineStr">
+        <is>
+          <t>sourceBasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1" s="15">
+      <c r="A51" s="39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B51" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="28" customHeight="1" s="15">
+      <c r="A52" s="39" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D52" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1" s="15">
+      <c r="A53" s="39" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B53" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D53" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1" s="15">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B54" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C54" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D54" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1" s="15">
+      <c r="A55" s="39" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B55" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D55" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1" s="15">
+      <c r="A56" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B56" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C56" s="39" t="inlineStr">
+        <is>
+          <t>EXTERNAL_OR_PERSONAL_CAUSE</t>
+        </is>
+      </c>
+      <c r="D56" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1; Dual existing divergence-map semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1" s="15">
+      <c r="A57" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B57" s="39" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C57" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D57" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1" s="15">
+      <c r="A58" s="39" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B58" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C58" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D58" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1" s="15">
+      <c r="A59" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B59" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C59" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D59" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1" s="15">
+      <c r="A60" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B60" s="39" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C60" s="39" t="inlineStr">
+        <is>
+          <t>STRUCTURAL_PRECONDITION_ABSENCE</t>
+        </is>
+      </c>
+      <c r="D60" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1" s="15">
+      <c r="A61" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B61" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C61" s="39" t="inlineStr">
+        <is>
+          <t>EVENT_ABSENCE</t>
+        </is>
+      </c>
+      <c r="D61" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1" s="15">
+      <c r="A62" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B62" s="39" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C62" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D62" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="15">
+      <c r="A63" s="39" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B63" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C63" s="39" t="inlineStr">
+        <is>
+          <t>AMBIGUOUS_COLLAPSE</t>
+        </is>
+      </c>
+      <c r="D63" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1; X-2 preserved, not repaired</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" s="15">
+      <c r="A64" s="39" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B64" s="39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C64" s="39" t="inlineStr">
+        <is>
+          <t>SUBSTANTIVE_SIGNAL</t>
+        </is>
+      </c>
+      <c r="D64" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1; Dual 1 Q11-E is a substantive environment signal, not an abstention</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1" s="15">
+      <c r="A65" s="39" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B65" s="39" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C65" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="D65" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted question-qualified E/F table D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="37" t="inlineStr">
+        <is>
+          <t>BLOCK C2 — Semantic_Class_Effects</t>
+        </is>
+      </c>
+      <c r="B67" s="40" t="n"/>
+      <c r="C67" s="40" t="n"/>
+      <c r="D67" s="40" t="n"/>
+      <c r="E67" s="40" t="n"/>
+      <c r="F67" s="41" t="n"/>
+    </row>
+    <row r="68" ht="22" customHeight="1" s="15">
+      <c r="A68" s="38" t="inlineStr">
+        <is>
+          <t>semanticClass</t>
+        </is>
+      </c>
+      <c r="B68" s="38" t="inlineStr">
+        <is>
+          <t>useClassEffect</t>
+        </is>
+      </c>
+      <c r="C68" s="38" t="inlineStr">
+        <is>
+          <t>signalEffect</t>
+        </is>
+      </c>
+      <c r="D68" s="38" t="inlineStr">
+        <is>
+          <t>coverageEffect</t>
+        </is>
+      </c>
+      <c r="E68" s="38" t="inlineStr">
+        <is>
+          <t>rootCauseFamily</t>
+        </is>
+      </c>
+      <c r="F68" s="38" t="inlineStr">
+        <is>
+          <t>sourceBasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="36" customHeight="1" s="15">
+      <c r="A69" s="39" t="inlineStr">
+        <is>
+          <t>OBSERVATION_GAP</t>
+        </is>
+      </c>
+      <c r="B69" s="39" t="inlineStr">
+        <is>
+          <t>comparable answer unavailable; excluded from ordinary comparison</t>
+        </is>
+      </c>
+      <c r="C69" s="39" t="inlineStr">
+        <is>
+          <t>no comparable environment signal</t>
+        </is>
+      </c>
+      <c r="D69" s="39" t="inlineStr">
+        <is>
+          <t>coverage gap</t>
+        </is>
+      </c>
+      <c r="E69" s="39" t="inlineStr">
+        <is>
+          <t>RC-B</t>
+        </is>
+      </c>
+      <c r="F69" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted semantic class effects D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="36" customHeight="1" s="15">
+      <c r="A70" s="39" t="inlineStr">
+        <is>
+          <t>EVENT_ABSENCE</t>
+        </is>
+      </c>
+      <c r="B70" s="39" t="inlineStr">
+        <is>
+          <t>comparable substantive answer unavailable; excluded</t>
+        </is>
+      </c>
+      <c r="C70" s="39" t="inlineStr">
+        <is>
+          <t>diagnostic finding; NOT an evidence penalty</t>
+        </is>
+      </c>
+      <c r="D70" s="39" t="inlineStr">
+        <is>
+          <t>excluded; not a quality penalty</t>
+        </is>
+      </c>
+      <c r="E70" s="39" t="inlineStr">
+        <is>
+          <t>RC-C</t>
+        </is>
+      </c>
+      <c r="F70" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted semantic class effects D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="36" customHeight="1" s="15">
+      <c r="A71" s="39" t="inlineStr">
+        <is>
+          <t>STRUCTURAL_PRECONDITION_ABSENCE</t>
+        </is>
+      </c>
+      <c r="B71" s="39" t="inlineStr">
+        <is>
+          <t>comparable substantive answer unavailable; excluded</t>
+        </is>
+      </c>
+      <c r="C71" s="39" t="inlineStr">
+        <is>
+          <t>diagnostic finding; NOT an evidence penalty</t>
+        </is>
+      </c>
+      <c r="D71" s="39" t="inlineStr">
+        <is>
+          <t>excluded; not a quality penalty</t>
+        </is>
+      </c>
+      <c r="E71" s="39" t="inlineStr">
+        <is>
+          <t>RC-C</t>
+        </is>
+      </c>
+      <c r="F71" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted semantic class effects D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="36" customHeight="1" s="15">
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>EXTERNAL_OR_PERSONAL_CAUSE</t>
+        </is>
+      </c>
+      <c r="B72" s="39" t="inlineStr">
+        <is>
+          <t>not globally treated as access gap</t>
+        </is>
+      </c>
+      <c r="C72" s="39" t="inlineStr">
+        <is>
+          <t>no environment signal; preserve existing Dual divergence-map semantics</t>
+        </is>
+      </c>
+      <c r="D72" s="39" t="inlineStr">
+        <is>
+          <t>not a global coverage-gap class</t>
+        </is>
+      </c>
+      <c r="E72" s="39" t="inlineStr">
+        <is>
+          <t>existing Dual Q6-E semantics</t>
+        </is>
+      </c>
+      <c r="F72" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted semantic class effects D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="36" customHeight="1" s="15">
+      <c r="A73" s="39" t="inlineStr">
+        <is>
+          <t>AMBIGUOUS_COLLAPSE</t>
+        </is>
+      </c>
+      <c r="B73" s="39" t="inlineStr">
+        <is>
+          <t>comparable answer unavailable; preserve ambiguity</t>
+        </is>
+      </c>
+      <c r="C73" s="39" t="inlineStr">
+        <is>
+          <t>do not resolve; reference X-2</t>
+        </is>
+      </c>
+      <c r="D73" s="39" t="inlineStr">
+        <is>
+          <t>do NOT resolve RC-B vs RC-C mechanically</t>
+        </is>
+      </c>
+      <c r="E73" s="39" t="inlineStr">
+        <is>
+          <t>unresolved (X-2)</t>
+        </is>
+      </c>
+      <c r="F73" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted semantic class effects D0_R1; X-2 preserved</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="36" customHeight="1" s="15">
+      <c r="A74" s="39" t="inlineStr">
+        <is>
+          <t>SUBSTANTIVE_SIGNAL</t>
+        </is>
+      </c>
+      <c r="B74" s="39" t="inlineStr">
+        <is>
+          <t>normal UseClass determination</t>
+        </is>
+      </c>
+      <c r="C74" s="39" t="inlineStr">
+        <is>
+          <t>normal environment signal mapping from Dual 1</t>
+        </is>
+      </c>
+      <c r="D74" s="39" t="inlineStr">
+        <is>
+          <t>not an abstention</t>
+        </is>
+      </c>
+      <c r="E74" s="39" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F74" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted semantic class effects D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="37" t="inlineStr">
+        <is>
+          <t>BLOCK C3 — Actual_Access_Ceiling</t>
+        </is>
+      </c>
+      <c r="B76" s="40" t="n"/>
+      <c r="C76" s="40" t="n"/>
+      <c r="D76" s="40" t="n"/>
+      <c r="E76" s="41" t="n"/>
+    </row>
+    <row r="77" ht="22" customHeight="1" s="15">
+      <c r="A77" s="38" t="inlineStr">
+        <is>
+          <t>signal</t>
+        </is>
+      </c>
+      <c r="B77" s="38" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C77" s="38" t="inlineStr">
+        <is>
+          <t>useClassCeiling</t>
+        </is>
+      </c>
+      <c r="D77" s="38" t="inlineStr">
+        <is>
+          <t>rootCauseFamily</t>
+        </is>
+      </c>
+      <c r="E77" s="38" t="inlineStr">
+        <is>
+          <t>sourceBasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="36" customHeight="1" s="15">
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t>directObservationGate</t>
+        </is>
+      </c>
+      <c r="B78" s="39" t="inlineStr">
+        <is>
+          <t>no + substantive option</t>
+        </is>
+      </c>
+      <c r="C78" s="39" t="inlineStr">
+        <is>
+          <t>CONTEXTUAL</t>
+        </is>
+      </c>
+      <c r="D78" s="39" t="inlineStr">
+        <is>
+          <t>RC-B</t>
+        </is>
+      </c>
+      <c r="E78" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted global actual access rules D0_R1; DEC-4 (per-answer factual signal, not accessLevel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="36" customHeight="1" s="15">
+      <c r="A79" s="39" t="inlineStr">
+        <is>
+          <t>evidenceType</t>
+        </is>
+      </c>
+      <c r="B79" s="39" t="inlineStr">
+        <is>
+          <t>hypothetical</t>
+        </is>
+      </c>
+      <c r="C79" s="39" t="inlineStr">
+        <is>
+          <t>CONTEXTUAL</t>
+        </is>
+      </c>
+      <c r="D79" s="39" t="inlineStr">
+        <is>
+          <t>RC-B</t>
+        </is>
+      </c>
+      <c r="E79" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted global actual access rules D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="36" customHeight="1" s="15">
+      <c r="A80" s="39" t="inlineStr">
+        <is>
+          <t>evidenceType</t>
+        </is>
+      </c>
+      <c r="B80" s="39" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C80" s="39" t="inlineStr">
+        <is>
+          <t>n/a — comparable answer unavailable</t>
+        </is>
+      </c>
+      <c r="D80" s="39" t="inlineStr">
+        <is>
+          <t>RC-B</t>
+        </is>
+      </c>
+      <c r="E80" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted global actual access rules D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="36" customHeight="1" s="15">
+      <c r="A81" s="39" t="inlineStr">
+        <is>
+          <t>roleCode</t>
+        </is>
+      </c>
+      <c r="B81" s="39" t="inlineStr">
+        <is>
+          <t>unspecified</t>
+        </is>
+      </c>
+      <c r="C81" s="39" t="inlineStr">
+        <is>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="D81" s="39" t="inlineStr">
+        <is>
+          <t>practitioner access review</t>
+        </is>
+      </c>
+      <c r="E81" s="39" t="inlineStr">
+        <is>
+          <t>Owner-accepted global actual access rules D0_R1; controlling question rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="72" customHeight="1" s="15">
+      <c r="A83" s="36" t="inlineStr">
+        <is>
+          <t>No global E → observation gap or F → event absence rule. E/F are questionRef + optionCode only (C1). accessLevel remains respondent-wide metadata for routing / analyst review / anomaly detection; it is not a multiplier, not an automatic UseClass, and not a global per-question cap. No new Schema field. A structural access issue must not be independently scored through UseClass AND speaks_for_group_without_access AND forced inference AND overgeneralized AND reliability as multiple causal penalties (target rule; X-3 S-1/S-2 not physically closed). No lie-detection / deception / demeanor inference language.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="10">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="A83:F83"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2010,7 +3785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="15" min="1" max="1"/>
@@ -2026,14 +3801,14 @@
     <row r="1" ht="28" customHeight="1" s="15">
       <c r="A1" s="35" t="inlineStr">
         <is>
-          <t>CLASSIFICATION PRECEDENCE · sole canonical evaluation-order authority · v3.1 D0_R0</t>
+          <t>CLASSIFICATION PRECEDENCE · sole canonical evaluation-order authority · v3.1 D0_R1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="96" customHeight="1" s="15">
       <c r="A2" s="36" t="inlineStr">
         <is>
-          <t>Priorities are evaluated strictly in order. The first matching priority terminates evaluation. Priorities 0a, 0b, 1, and 1b are precondition / coverage outcomes. They may stop the five-state classifier. They are NOT divergence states and MUST NOT appear in the divergence-state enum. The divergence-state enum contains exactly five members: ① CONVERGENT, ② PARTIAL CONVERGENCE, ③ ROLE-LEVEL SPLIT, ④-A IRRESOLVABLE — within-pair divergence, ④-B IRRESOLVABLE — pair-identification failure. Sheet 7 is an override / pre-classification layer, not a parallel state table. Where sheet 7 and sheet 5 could both apply, this sheet governs. This comparator never emits a final Environment label.</t>
+          <t>Priorities are evaluated strictly in order. The first matching priority terminates evaluation. Priorities 0a, 0b, 0c, 1, 1b, and 3a are input / coverage / routing outcomes. They may stop the five-state classifier. They are NOT divergence states and MUST NOT appear in the divergence-state enum. The divergence-state enum contains exactly five members: ① CONVERGENT, ② PARTIAL CONVERGENCE, ③ ROLE-LEVEL SPLIT, ④-A IRRESOLVABLE — within-pair divergence, ④-B IRRESOLVABLE — pair-identification failure. Sheet 7 is an override / pre-classification layer, not a parallel state table. Where sheet 7 and sheet 5 could both apply, this sheet governs. This comparator never emits a final Environment label. MATERIALIZED METHODOLOGY / GENERATED CORPUS is not PRODUCTION-ACTIVE OBSERVATION SCOPE; production-active Observation Scope remains blocked by X-3 S-1/S-2.</t>
         </is>
       </c>
     </row>
@@ -2159,53 +3934,57 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" s="15">
+    <row r="7" ht="72" customHeight="1" s="15">
       <c r="A7" s="39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0c</t>
         </is>
       </c>
       <c r="B7" s="39" t="inlineStr">
         <is>
-          <t>Combined evidence-quality multiplier &lt; 0.4 on ≥ 8 of 11 questions OR both respondents answered E to both HIGH-weight pair resolvers</t>
+          <t>Required eligibility UNRESOLVED (including roleCode = unspecified, or external default UseClass UNRESOLVED)</t>
         </is>
       </c>
       <c r="C7" s="39" t="inlineStr">
         <is>
-          <t>coverage_outcome</t>
+          <t>routing_outcome</t>
         </is>
       </c>
       <c r="D7" s="39" t="inlineStr">
         <is>
-          <t>COVERAGE INSUFFICIENT — comparator output suppressed</t>
+          <t>Practitioner access review</t>
         </is>
       </c>
       <c r="E7" s="39" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F7" s="39" t="n"/>
+          <t>Yes — detect</t>
+        </is>
+      </c>
+      <c r="F7" s="39" t="inlineStr">
+        <is>
+          <t>Practitioner access review</t>
+        </is>
+      </c>
       <c r="G7" s="39" t="inlineStr">
         <is>
-          <t>No signal pattern; no Contradiction records</t>
+          <t>No five-state classification; no Contradiction record from this comparator</t>
         </is>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
-          <t>DR-C2; DR-C6; C-21</t>
+          <t>DEC-4; controlling question rules</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1" s="15">
       <c r="A8" s="39" t="inlineStr">
         <is>
-          <t>1b</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B8" s="39" t="inlineStr">
         <is>
-          <t>Both respondents answered F to Q11</t>
+          <t>Branch (i): ≥ 8 of 11 questions have PRIMARY × PRIMARY comparable comparison unavailable OR provisional PRIMARY × PRIMARY four-factor &lt; 0.4 (number 8/11 unchanged; DEC-8 PRIMARY × CONTEXTUAL state-③ check is NOT counted). Branch (ii): both respondents lack a comparable PRIMARY answer on all HIGH resolvers defined for the active pair (HIGH cardinality from sheet 2). Branch (iii): a defined HIGH resolver is not PRIMARY for both respondents (DEC-3) — coverage/routing outcome, not ①/④-A.</t>
         </is>
       </c>
       <c r="C8" s="39" t="inlineStr">
@@ -2215,81 +3994,77 @@
       </c>
       <c r="D8" s="39" t="inlineStr">
         <is>
-          <t>NF/SFP determination impossible</t>
+          <t>COVERAGE INSUFFICIENT — comparator output suppressed</t>
         </is>
       </c>
       <c r="E8" s="39" t="inlineStr">
         <is>
-          <t>Yes — detect</t>
-        </is>
-      </c>
-      <c r="F8" s="39" t="inlineStr">
-        <is>
-          <t>Practitioner review</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F8" s="39" t="n"/>
       <c r="G8" s="39" t="inlineStr">
         <is>
-          <t>Pair evaluation suppressed for NF/SFP vs NF/SFJ / Q11 discriminator family; no automatic EDv2 fallback</t>
+          <t>No signal pattern; no Contradiction records</t>
         </is>
       </c>
       <c r="H8" s="39" t="inlineStr">
         <is>
-          <t>DR-A6; DR-C6</t>
+          <t>DR-C2; DR-C6; C-21</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1" s="15">
       <c r="A9" s="39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1b</t>
         </is>
       </c>
       <c r="B9" s="39" t="inlineStr">
         <is>
-          <t>Evidence concentrates on an environment OUTSIDE the candidate pair, at quality ≥ 0.5</t>
+          <t>Both respondents Q11 = F (OBSERVATION_GAP) / NF/SFP determination impossible; or equivalent UseClass unavailability on Q11 for the NF/SFP vs NF/SFJ pair / Q11 discriminator family. Q11 E is SUBSTANTIVE_SIGNAL and is not an abstention.</t>
         </is>
       </c>
       <c r="C9" s="39" t="inlineStr">
         <is>
-          <t>divergence_state</t>
+          <t>coverage_outcome</t>
         </is>
       </c>
       <c r="D9" s="39" t="inlineStr">
         <is>
-          <t>Candidate ④-B — pair-identification failure</t>
+          <t>NF/SFP determination impossible</t>
         </is>
       </c>
       <c r="E9" s="39" t="inlineStr">
         <is>
-          <t>Detect only</t>
+          <t>Yes — detect</t>
         </is>
       </c>
       <c r="F9" s="39" t="inlineStr">
         <is>
-          <t>Practitioner confirmation required</t>
+          <t>Practitioner review</t>
         </is>
       </c>
       <c r="G9" s="39" t="inlineStr">
         <is>
-          <t>After confirmation: BLOCKED; 1 critical Contradiction record, contradictionType = cross_respondent_same_side</t>
+          <t>Pair evaluation suppressed for NF/SFP vs NF/SFJ / Q11 discriminator family; no automatic EDv2 fallback</t>
         </is>
       </c>
       <c r="H9" s="39" t="inlineStr">
         <is>
-          <t>DR-C2; DR-C4; DR-D5</t>
+          <t>DR-A6; DR-C6</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1" s="15">
       <c r="A10" s="39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B10" s="39" t="inlineStr">
         <is>
-          <t>BOTH HIGH-weight pair resolvers DIVERGE at quality ≥ 0.5</t>
+          <t>Evidence concentrates on an environment OUTSIDE the candidate pair, at quality ≥ 0.5</t>
         </is>
       </c>
       <c r="C10" s="39" t="inlineStr">
@@ -2299,115 +4074,119 @@
       </c>
       <c r="D10" s="39" t="inlineStr">
         <is>
-          <t>④-A IRRESOLVABLE — within-pair divergence</t>
+          <t>Candidate ④-B — pair-identification failure</t>
         </is>
       </c>
       <c r="E10" s="39" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F10" s="39" t="n"/>
+          <t>Detect only</t>
+        </is>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>Practitioner confirmation required</t>
+        </is>
+      </c>
       <c r="G10" s="39" t="inlineStr">
         <is>
-          <t>BLOCKED; 1 high Contradiction record</t>
+          <t>After confirmation: BLOCKED; 1 critical Contradiction record, contradictionType = cross_respondent_same_side</t>
         </is>
       </c>
       <c r="H10" s="39" t="inlineStr">
         <is>
-          <t>DR-C2; DR-C3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1" s="15">
+          <t>DR-C2; DR-C4; DR-D5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1" s="15">
       <c r="A11" s="39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3a</t>
         </is>
       </c>
       <c r="B11" s="39" t="inlineStr">
         <is>
-          <t>AGREE on ≥ 5 non-governance axes AND DIVERGE on Q1 and/or Q5 AND one respondent is senior-tier and the other line-level tier; quality ≥ 0.5</t>
+          <t>Active pair = NF/SFP vs NF/SFJ (canonical one-HIGH; sole HIGH = Q11); Q11 DIVERGE; Q11 PRIMARY × PRIMARY; provisional four-factor ≥ 0.5</t>
         </is>
       </c>
       <c r="C11" s="39" t="inlineStr">
         <is>
-          <t>divergence_state</t>
+          <t>routing_outcome</t>
         </is>
       </c>
       <c r="D11" s="39" t="inlineStr">
         <is>
-          <t>③ ROLE-LEVEL SPLIT</t>
+          <t>Practitioner review — one-HIGH coverage insufficient for automatic ④-A</t>
         </is>
       </c>
       <c r="E11" s="39" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F11" s="39" t="n"/>
+          <t>Yes — detect</t>
+        </is>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>Practitioner review</t>
+        </is>
+      </c>
       <c r="G11" s="39" t="inlineStr">
         <is>
-          <t>★ WEAK signal pattern + SPLIT annotation; 1 medium Contradiction record; standard analyst review queue; NO Gate 4</t>
+          <t>NOT ④-A. No automatic high-severity Contradiction Record. No new divergence state. No new contradictionType.</t>
         </is>
       </c>
       <c r="H11" s="39" t="inlineStr">
         <is>
-          <t>DR-C2; DR-B4</t>
+          <t>DEC-7; X-9</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1" s="15">
       <c r="A12" s="39" t="inlineStr">
         <is>
-          <t>5X</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B12" s="39" t="inlineStr">
         <is>
-          <t>①/② agreement-count criteria satisfied but agreement environment coherence is ambiguous</t>
+          <t>All HIGH resolvers defined for the active pair DIVERGE at PRIMARY × PRIMARY with provisional four-factor ≥ 0.5 (after 3a has intercepted the canonical one-HIGH pair)</t>
         </is>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>routing_outcome</t>
+          <t>divergence_state</t>
         </is>
       </c>
       <c r="D12" s="39" t="inlineStr">
         <is>
-          <t>ANALYST / PRACTITIONER REVIEW — no automatic state</t>
+          <t>④-A IRRESOLVABLE — within-pair divergence</t>
         </is>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
-          <t>Detect only</t>
-        </is>
-      </c>
-      <c r="F12" s="39" t="inlineStr">
-        <is>
-          <t>Analyst / practitioner review</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F12" s="39" t="n"/>
       <c r="G12" s="39" t="inlineStr">
         <is>
-          <t>Held pending review; MUST NOT auto-classify as ④-B</t>
+          <t>BLOCKED; 1 high Contradiction record</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>DR-C5</t>
+          <t>DR-C2; DR-C3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1" s="15">
       <c r="A13" s="39" t="inlineStr">
         <is>
-          <t>5A</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B13" s="39" t="inlineStr">
         <is>
-          <t>Effective AGREE ≥ 7 of 11; both HIGH-weight pair resolvers agree; quality ≥ 0.7</t>
+          <t>Exactly one senior-tier and one line_level-tier; Q1 and/or Q5 materially DIVERGE (senior PRIMARY × line-level CONTEXTUAL); DEC-8 triggering four-factor ≥ 0.5 on those questions (quality-admissibility only); ≥ 5 non-governance PRIMARY × PRIMARY AGREE each with provisional four-factor ≥ 0.5</t>
         </is>
       </c>
       <c r="C13" s="39" t="inlineStr">
@@ -2417,7 +4196,7 @@
       </c>
       <c r="D13" s="39" t="inlineStr">
         <is>
-          <t>① CONVERGENT</t>
+          <t>③ ROLE-LEVEL SPLIT</t>
         </is>
       </c>
       <c r="E13" s="39" t="inlineStr">
@@ -2428,48 +4207,128 @@
       <c r="F13" s="39" t="n"/>
       <c r="G13" s="39" t="inlineStr">
         <is>
-          <t>★★★ STRONG signal pattern; 0 Contradiction records</t>
+          <t>★ WEAK signal pattern + SPLIT annotation; 1 medium Contradiction record; standard analyst review queue; NO Gate 4</t>
         </is>
       </c>
       <c r="H13" s="39" t="inlineStr">
         <is>
-          <t>DR-C2</t>
+          <t>DR-C2; DR-B4</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1" s="15">
       <c r="A14" s="39" t="inlineStr">
         <is>
+          <t>5X</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>①/② agreement-count criteria satisfied but agreement environment coherence is ambiguous</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>routing_outcome</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="inlineStr">
+        <is>
+          <t>ANALYST / PRACTITIONER REVIEW — no automatic state</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>Detect only</t>
+        </is>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>Analyst / practitioner review</t>
+        </is>
+      </c>
+      <c r="G14" s="39" t="inlineStr">
+        <is>
+          <t>Held pending review; MUST NOT auto-classify as ④-B</t>
+        </is>
+      </c>
+      <c r="H14" s="39" t="inlineStr">
+        <is>
+          <t>DR-C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>Effective AGREE ≥ 7 PRIMARY × PRIMARY; all HIGH resolvers defined for the active pair AGREE and are PRIMARY for both; provisional four-factor ≥ 0.7</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>divergence_state</t>
+        </is>
+      </c>
+      <c r="D15" s="39" t="inlineStr">
+        <is>
+          <t>① CONVERGENT</t>
+        </is>
+      </c>
+      <c r="E15" s="39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" s="39" t="n"/>
+      <c r="G15" s="39" t="inlineStr">
+        <is>
+          <t>★★★ STRONG signal pattern; 0 Contradiction records</t>
+        </is>
+      </c>
+      <c r="H15" s="39" t="inlineStr">
+        <is>
+          <t>DR-C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
           <t>5B</t>
         </is>
       </c>
-      <c r="B14" s="39" t="inlineStr">
-        <is>
-          <t>Effective AGREE 5–6 of 11; at least one HIGH-weight pair resolver agrees; quality ≥ 0.5</t>
-        </is>
-      </c>
-      <c r="C14" s="39" t="inlineStr">
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>Effective AGREE 5–6 PRIMARY × PRIMARY; at least one defined HIGH resolver AGREES and is PRIMARY for both; provisional four-factor ≥ 0.5. DEC-7b: one-HIGH pair still requires this 5–6 floor.</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>divergence_state</t>
         </is>
       </c>
-      <c r="D14" s="39" t="inlineStr">
+      <c r="D16" s="39" t="inlineStr">
         <is>
           <t>② PARTIAL CONVERGENCE</t>
         </is>
       </c>
-      <c r="E14" s="39" t="inlineStr">
+      <c r="E16" s="39" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="39" t="n"/>
-      <c r="G14" s="39" t="inlineStr">
+      <c r="F16" s="39" t="n"/>
+      <c r="G16" s="39" t="inlineStr">
         <is>
           <t>★★ CONFIRMED signal pattern; 0–3 Contradiction records</t>
         </is>
       </c>
-      <c r="H14" s="39" t="inlineStr">
+      <c r="H16" s="39" t="inlineStr">
         <is>
           <t>DR-C2</t>
         </is>
@@ -5071,7 +6930,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1" s="15">
+    <row r="2" ht="180" customHeight="1" s="15">
       <c r="A2" s="17" t="inlineStr">
         <is>
           <t>CANDIDATE-PAIR CONTRACT (v3.1, corrected).
@@ -5080,7 +6939,8 @@
 3. Pair orientation. A candidate pair is an unordered identity. AGREE/DIVERGE logic applies symmetrically under reversal of the two respondents. Respondent identities R1 and R2 are nonetheless retained throughout. The single exception where respondent identity/role is a load-bearing semantic input is state ③ ROLE-LEVEL SPLIT (sheet 5).
 4. Unsupported pairs. If the supplied candidatePair is not one of the five above: STOP — practitioner pair diagnosis required. This is an input/precondition failure, NOT ④-B. No default weights, no fallback weights, and no generic invented weights may be created for any pair outside this set.
 5. Q11 discriminator family. NF/SFP vs other is NOT a sixth candidate pair. It is the Q11 discriminator / complement family, recorded on sheet 3: option C = NF/SFP signal branch, options A/B/D/E = non-NF/SFP signal branch. other is never a canonical Environment and never a pair identity. For the concrete pair NF/SFP vs NF/SFJ, the specific pair rows on this sheet take precedence over the complement-family rule.
-6. Product boundary. This comparator produces a divergence state and a signal pattern. It never produces, resolves, or merges a final Environment label.</t>
+6. Product boundary. This comparator produces a divergence state and a signal pattern. It never produces, resolves, or merges a final Environment label.
+7. HIGH-resolver cardinality (X-9). Pair-specific weight rows on this sheet are the controlling source. HIGH-resolver cardinality is defined per pair from those rows. Four production pairs have two HIGH resolvers. NF/SFP vs NF/SFJ has exactly one HIGH resolver: Q11. Q11 is the sole NF/SFP discriminator. No second HIGH resolver is inferred or assigned (Q10 on this pair remains STANDARD).</t>
         </is>
       </c>
     </row>
@@ -6096,7 +7956,7 @@
       </c>
       <c r="G5" s="32" t="inlineStr">
         <is>
-          <t>STANDARD (HIGH for STJ/STP vs NT/STJ pair when R1=A R2=C)</t>
+          <t>STANDARD (sheet 2 controlling; Q1 is STANDARD for all listed pairs; not HIGH)</t>
         </is>
       </c>
       <c r="H5" s="32" t="inlineStr">
@@ -6180,7 +8040,7 @@
       </c>
       <c r="G7" s="32" t="inlineStr">
         <is>
-          <t>HIGH (NF/SFJ vs NF/NT)</t>
+          <t>STANDARD (sheet 2 controlling; Q3 is STANDARD for NF/SFJ vs NF/NT; not HIGH)</t>
         </is>
       </c>
       <c r="H7" s="32" t="inlineStr">
@@ -6264,7 +8124,7 @@
       </c>
       <c r="G9" s="32" t="inlineStr">
         <is>
-          <t>HIGH (NT/STJ vs NT/STP and SFJ/SFP vs SFP/SFJ)</t>
+          <t>STANDARD (sheet 2 controlling; Q5 is STANDARD for listed pairs; not HIGH)</t>
         </is>
       </c>
       <c r="H9" s="32" t="inlineStr">
@@ -6562,7 +8422,7 @@
     <row r="2" ht="109.5" customHeight="1" s="15">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>NEW IN v3.1. The pre-rebuild source applied uniform weight to every divergence. v3.1 weights divergence by evidence-machinery quality: a divergence between two direct-observation answers from senior-tier respondents with high confidence and zero reliability flags is high-quality evidence for an analyst contradiction. A divergence between two inference-based answers from line-level-tier respondents with multiple reliability flags is low-quality and should NOT trigger a contradiction record without analyst escalation.</t>
+          <t>DEC-1. Role coverage is removed from evidence-quality multiplication. Observation Use Class (sheet 11) governs admissibility; seniority is not an evidence-quality score. Ordinary structural comparison uses a PROVISIONAL FOUR-FACTOR PRODUCT (evidenceType × knowledgeLevel × confidence × reliabilityFlags) on PRIMARY × PRIMARY only. Status: PROVISIONAL — PENDING C-25/X-4. Existing thresholds 0.7 / 0.5 / 0.4 / 0.2 are retained; not recalibrated. DEC-8: a separate PRIMARY × CONTEXTUAL four-factor check (≥ 0.5) applies only as a quality-admissibility gate on triggering Q1/Q5 for state ③. That check is not a structural resolver score and is not counted in priority-1 coverage.</t>
         </is>
       </c>
     </row>
@@ -6711,68 +8571,68 @@
     <row r="10" ht="78" customHeight="1" s="15">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>Role-coverage match</t>
+          <t>Role-coverage match — SUPERSEDED BY OBSERVATION SCOPE LAYER — DEC-1</t>
         </is>
       </c>
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>Both respondents are within legitimate observation scope for this question per sheet 11_Role_Question_Scope of this workbook. ST_Canonical_Schema.xlsx v1.1 sheet 14_RoleCoverageMatrix is a deal-size respondent-coverage tier rule and is NOT a role × question observation-scope matrix.</t>
+          <t>SUPERSEDED BY OBSERVATION SCOPE LAYER — DEC-1. Historical high-quality condition retained for audit: Both respondents are within legitimate observation scope for this question per sheet 11_Role_Question_Scope of this workbook. ST_Canonical_Schema.xlsx v1.1 sheet 14_RoleCoverageMatrix is a deal-size respondent-coverage tier rule and is NOT a role × question observation-scope matrix.</t>
         </is>
       </c>
       <c r="C10" s="32" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>SUPERSEDED — not a multiplicative factor. Historical cell: 1.0</t>
         </is>
       </c>
       <c r="D10" s="32" t="inlineStr">
         <is>
-          <t>Either respondent is below-tier for this question scope (e.g. line-level-tier respondent answering Axis 1 questions)</t>
+          <t>SUPERSEDED. Historical low-quality condition retained for audit: Either respondent is below-tier for this question scope (e.g. line-level-tier respondent answering Axis 1 questions)</t>
         </is>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
-          <t>Apply 0.5 multiplier; route to ROLE-LEVEL SPLIT classification (sheet 5 state ③) if pattern is systematic. Dimension 5 is NOT production-ready until sheet 11_Role_Question_Scope is authored and accepted. No default, fallback, or 1.0 substitution for a missing roleCoverageMultiplier is permitted. Until then the five-factor combined-quality model is INCOMPLETE.</t>
+          <t>SUPERSEDED BY OBSERVATION SCOPE LAYER — DEC-1. Not used in the provisional four-factor product. Historical action retained for audit: Apply 0.5 multiplier; route to ROLE-LEVEL SPLIT classification (sheet 5 state ③) if pattern is systematic. Dimension 5 is NOT production-ready until sheet 11_Role_Question_Scope is authored and accepted. No default, fallback, or 1.0 substitution for a missing roleCoverageMultiplier is permitted. Until then the five-factor combined-quality model is INCOMPLETE.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="78" customHeight="1" s="15">
       <c r="A11" s="33" t="inlineStr">
         <is>
-          <t>Combined quality multiplier</t>
+          <t>Provisional four-factor product</t>
         </is>
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>Product of all 5 dimension multipliers</t>
+          <t>PROVISIONAL FOUR-FACTOR PRODUCT for ordinary structural comparison (PRIMARY × PRIMARY): evidenceType × knowledgeLevel × confidence × reliabilityFlags. Role-coverage is not a factor. PROVISIONAL — PENDING C-25/X-4.</t>
         </is>
       </c>
       <c r="C11" s="34" t="inlineStr">
         <is>
-          <t>Range: 0.027 to 1.0</t>
+          <t>SUPERSEDED / ANNULLED — NO REPLACEMENT RANGE PENDING C-25/X-4</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
         <is>
-          <t>Below 0.4 = low-quality divergence; below 0.2 = excluded entirely</t>
+          <t>Below 0.4 = low-quality divergence; below 0.2 = excluded entirely. Thresholds 0.7 / 0.5 / 0.4 / 0.2 retained; not recalibrated.</t>
         </is>
       </c>
       <c r="E11" s="34" t="inlineStr">
         <is>
-          <t>Multiplier ≥ 0.7: standard divergence weight applied. Multiplier 0.4-0.7: divergence flagged but reduced. Multiplier &lt; 0.4: divergence noted, NO Contradiction record produced.</t>
+          <t>Ordinary domain PRIMARY × PRIMARY: multiplier ≥ 0.7 standard divergence weight; 0.4–0.7 flagged but reduced; &lt; 0.4 noted, NO Contradiction record. DEC-8 domain PRIMARY × CONTEXTUAL on triggering Q1/Q5 is a separate state-③ quality-admissibility check only (≥ 0.5), OWNER-ADOPTED CORRECTION — PROVISIONAL, PENDING C-25/X-4. DEC-8 is not a structural resolver score, not AGREE/DIVERGE tally, not HIGH-resolver logic, and not priority-1 coverage.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="15">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>INTEGRATION WITH SHEET 3</t>
+          <t>USE DOMAINS AND OBSERVATION-SCOPE APPLICATION ORDER</t>
         </is>
       </c>
     </row>
     <row r="14" ht="129.75" customHeight="1" s="15">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Each per-question divergence determination from sheet 3 is multiplied by the combined evidence-quality multiplier from this sheet. Effective divergence weight = base_weight × combined_quality_multiplier. Sheet 5 (Divergence Classification) consumes the effective weights, NOT the base weights. This means a CONVERGENT classification requires both AGREE pattern AND high-quality evidence on enough questions; an IRRESOLVABLE classification can result from genuine cross-respondent divergence OR from systematically low-quality evidence.</t>
+          <t>Domain 1 — ordinary structural comparison: PRIMARY × PRIMARY only; provisional four-factor product. Domain 2 — state ③ triggering quality-admissibility check only: PRIMARY × CONTEXTUAL on triggering Q1/Q5; provisional four-factor ≥ 0.5; OWNER-ADOPTED CORRECTION — PROVISIONAL, PENDING C-25/X-4; not mixed with Domain 1. Observation Use Class application order on sheet 11: C1 → C2 → C3. Former combined range 0.027 to 1.0 is SUPERSEDED / ANNULLED — NO REPLACEMENT RANGE PENDING C-25/X-4. This comparator never produces a final Environment label.</t>
         </is>
       </c>
     </row>
@@ -6815,7 +8675,7 @@
     <row r="2" ht="91.5" customHeight="1" s="15">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Input: per-question divergence (sheet 3) × evidence-quality multiplier (sheet 4). Output: one of five divergence states: ① CONVERGENT, ② PARTIAL CONVERGENCE, ③ ROLE-LEVEL SPLIT, ④-A IRRESOLVABLE — within-pair divergence, ④-B IRRESOLVABLE — pair-identification failure. ④-A is reached automatically ONLY when BOTH HIGH-weight pair resolvers DIVERGE at quality ≥ 0.5. Engine may detect evidence outside the candidate pair, but FINAL ④-B classification requires practitioner confirmation. Adding a third respondent does NOT resolve ④-B. COVERAGE INSUFFICIENT and NF/SFP determination impossible are precondition / coverage outcomes, not divergence states. This comparator never produces a final Environment label.</t>
+          <t>Input: Observation Use Class (sheet 11) then provisional four-factor evidence quality (sheet 4) then per-question divergence (sheet 3). Output: one of five divergence states: ① CONVERGENT, ② PARTIAL CONVERGENCE, ③ ROLE-LEVEL SPLIT, ④-A IRRESOLVABLE — within-pair divergence, ④-B IRRESOLVABLE — pair-identification failure. Ordinary AGREE/DIVERGE tallies use PRIMARY × PRIMARY only. HIGH-resolver conditions use all HIGH resolvers defined for the active pair on sheet 2, and only if PRIMARY for both respondents (DEC-3). ④-A is automatic only when all defined HIGH resolvers DIVERGE at PRIMARY × PRIMARY with provisional quality ≥ 0.5; the canonical one-HIGH pair NF/SFP vs NF/SFJ is intercepted by priority 3a (DEC-7) and is not auto-④-A. Engine may detect evidence outside the candidate pair, but FINAL ④-B requires practitioner confirmation. INELIGIBLE and UNRESOLVED do not create pair-identification failure. COVERAGE INSUFFICIENT, NF/SFP determination impossible, UNRESOLVED access, and one-HIGH Q11 routing are not divergence states. This comparator never produces a final Environment label.</t>
         </is>
       </c>
     </row>
@@ -6866,17 +8726,17 @@
       </c>
       <c r="B6" s="32" t="inlineStr">
         <is>
-          <t>Effective AGREE on ≥7 of 11 questions (was 7 of 10 in source v1.0; v3.1 adjusts for Q11)</t>
+          <t>Effective AGREE ≥ 7 among PRIMARY × PRIMARY comparable questions</t>
         </is>
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>BOTH HIGH-weight pair-resolvers AGREE</t>
+          <t>All HIGH resolvers defined for the active pair AGREE, and each is PRIMARY for both respondents (DEC-3)</t>
         </is>
       </c>
       <c r="D6" s="32" t="inlineStr">
         <is>
-          <t>Combined quality multiplier ≥ 0.7 on agreement-contributing questions</t>
+          <t>Provisional four-factor product ≥ 0.7 on agreement-contributing PRIMARY × PRIMARY questions</t>
         </is>
       </c>
       <c r="E6" s="32" t="inlineStr">
@@ -6898,17 +8758,17 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>Effective AGREE on 5–6 of 11 questions</t>
+          <t>Effective AGREE 5–6 among PRIMARY × PRIMARY comparable questions. DEC-7b: for NF/SFP vs NF/SFJ the ordinary 5–6 floor still applies; one agreeing Q11 HIGH does not replace it (sheet 7!D6 override does not apply to that pair).</t>
         </is>
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>AT LEAST ONE HIGH-weight pair-resolver AGREES</t>
+          <t>At least one HIGH resolver defined for the active pair AGREES, and that resolver is PRIMARY for both respondents (DEC-3)</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>Combined quality multiplier ≥ 0.5 on agreement-contributing questions</t>
+          <t>Provisional four-factor product ≥ 0.5 on agreement-contributing PRIMARY × PRIMARY questions</t>
         </is>
       </c>
       <c r="E7" s="26" t="inlineStr">
@@ -6930,7 +8790,7 @@
       </c>
       <c r="B8" s="32" t="inlineStr">
         <is>
-          <t>AGREE on ≥5 non-governance axes AND DIVERGE on Q1 and/or Q5 AND one respondent is senior-tier and the other line-level tier (per sheet 11 Seniority Tier Mapping).</t>
+          <t>Exactly one senior-tier and one line_level-tier respondent. Q1 and/or Q5 materially DIVERGE with senior side PRIMARY and line-level side CONTEXTUAL. Agreement foundation: ≥ 5 non-governance PRIMARY × PRIMARY AGREE, each with provisional four-factor ≥ 0.5.</t>
         </is>
       </c>
       <c r="C8" s="32" t="inlineStr">
@@ -6940,7 +8800,7 @@
       </c>
       <c r="D8" s="32" t="inlineStr">
         <is>
-          <t>Quality multiplier ≥ 0.5 (role mismatch reduces it but does not invalidate)</t>
+          <t>DEC-8 OWNER-ADOPTED CORRECTION — PROVISIONAL, PENDING C-25/X-4: on each triggering Q1/Q5 (PRIMARY × CONTEXTUAL) the provisional four-factor product must be ≥ 0.5 as a quality-admissibility check only. Not a structural resolver score; not AGREE/DIVERGE tally; not HIGH-resolver logic; not priority-1 coverage.</t>
         </is>
       </c>
       <c r="E8" s="32" t="inlineStr">
@@ -6962,17 +8822,17 @@
       </c>
       <c r="B9" s="34" t="inlineStr">
         <is>
-          <t>BOTH HIGH-weight pair-resolvers DIVERGE (e.g. {Q4-A, Q4-B} split AND {Q7-A, Q7-B} split for NT/STJ vs NT/STP pair)</t>
+          <t>All HIGH resolvers defined for the active pair DIVERGE, each PRIMARY for both respondents, provisional quality ≥ 0.5 (e.g. {Q4-A, Q4-B} split AND {Q7-A, Q7-B} split for NT/STJ vs NT/STP). Canonical one-HIGH pair NF/SFP vs NF/SFJ is intercepted by sheet 12 priority 3a (DEC-7) and is not auto-④-A.</t>
         </is>
       </c>
       <c r="C9" s="34" t="inlineStr">
         <is>
-          <t>Both pair-resolvers fail</t>
+          <t>All defined HIGH resolvers fail (PRIMARY × PRIMARY DIVERGE)</t>
         </is>
       </c>
       <c r="D9" s="34" t="inlineStr">
         <is>
-          <t>Quality multiplier ≥ 0.5 on the failing questions (genuine divergence, not low-quality artifact)</t>
+          <t>Provisional four-factor product ≥ 0.5 on the failing HIGH questions (genuine divergence, not low-quality artifact)</t>
         </is>
       </c>
       <c r="E9" s="34" t="inlineStr">
@@ -6994,7 +8854,7 @@
       </c>
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t>One respondent's signals concentrate on an environment OUTSIDE the candidate pair (unordered — either respondent).</t>
+          <t>One respondent's signals concentrate on an environment OUTSIDE the candidate pair (unordered — either respondent). INELIGIBLE and UNRESOLVED do not create pair-identification failure.</t>
         </is>
       </c>
       <c r="C10" s="34" t="inlineStr">
@@ -7643,7 +9503,7 @@
     <row r="2" ht="57.75" customHeight="1" s="15">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Override / pre-classification layer. Applied BEFORE the five-state classifier. NOT a parallel state table. Where these edge cases and sheet 5 could both apply, sheet 12_Classification_Precedence governs. v3.1 preserves source v1.0 edge cases plus adds Option E/F edge cases.</t>
+          <t>Override / pre-classification layer. Applied BEFORE the five-state classifier. NOT a parallel state table. Where these edge cases and sheet 5 could both apply, sheet 12_Classification_Precedence governs. v3.1 preserves source v1.0 edge cases plus adds Option E/F edge cases. UNRESOLVED Observation Use Class routes to practitioner access review (sheet 12 priority 0c). Read “both HIGH” / “HIGH-weight pair-resolvers” as all HIGH resolvers defined for the active pair (sheet 2). DEC-7b: 7!D6 override does not apply to canonical one-HIGH pair NF/SFP vs NF/SFJ.</t>
         </is>
       </c>
     </row>
@@ -7694,12 +9554,12 @@
     <row r="6" ht="78" customHeight="1" s="15">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>Both HIGH-weight agree but total &lt; 5</t>
+          <t>All defined HIGH resolvers agree but total PRIMARY × PRIMARY AGREE &lt; 5</t>
         </is>
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
-          <t>Both pair-resolver questions agree, but only 3-4 of remaining 9 agree</t>
+          <t>All HIGH resolvers defined for the active pair AGREE (PRIMARY both), but only 3–4 remaining PRIMARY × PRIMARY questions agree</t>
         </is>
       </c>
       <c r="C6" s="26" t="inlineStr">
@@ -7709,7 +9569,7 @@
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>Pair-resolvers are authoritative for the specific pair. Agreement on both overrides the 5/11 total threshold for this pair. Append: "High-weight pair confirmation with partial screening agreement"</t>
+          <t>For multi-HIGH pairs: pair-resolvers are authoritative for the specific pair. Agreement on all defined HIGH resolvers overrides the 5/11 total threshold for this pair. Append: "High-weight pair confirmation with partial screening agreement". DEC-7b: this override does NOT apply to the canonical one-HIGH pair NF/SFP vs NF/SFJ. State ② for that pair still requires the ordinary 5–6 PRIMARY × PRIMARY agreements. A single agreeing Q11 HIGH does not replace the confirmation floor. Number 5–6 is unchanged.</t>
         </is>
       </c>
     </row>
@@ -7731,7 +9591,7 @@
       </c>
       <c r="D7" s="32" t="inlineStr">
         <is>
-          <t>Split pair-resolver result removes the ability to cleanly lock the pair. Treat as single-resolver confirmation with reduced confidence. ④-A is NOT reachable here: automatic ④-A requires divergence of BOTH HIGH-weight pair resolvers.</t>
+          <t>Split pair-resolver result removes the ability to cleanly lock the pair. Treat as single-resolver confirmation with reduced confidence. ④-A is NOT reachable here: automatic ④-A requires divergence of all HIGH resolvers defined for the active pair (PRIMARY both). Canonical one-HIGH Q11 DIVERGE is intercepted by priority 3a (DEC-7), not ④-A.</t>
         </is>
       </c>
     </row>
@@ -7787,7 +9647,7 @@
       </c>
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t>BOTH respondents answered E to BOTH HIGH-weight pair-resolver questions</t>
+          <t>BOTH respondents answered E to all HIGH resolvers defined for the active pair</t>
         </is>
       </c>
       <c r="C10" s="34" t="inlineStr">
@@ -7797,7 +9657,7 @@
       </c>
       <c r="D10" s="34" t="inlineStr">
         <is>
-          <t>Pair-resolvers cannot be evaluated. This is absence of evidence, not genuine divergence. Under the canonical ④-A rule, ④-A is reachable ONLY when both HIGH-weight pair resolvers DIVERGE at quality ≥ 0.5. No Contradiction record is emitted. Practitioner may consider supplemental respondents or interview.</t>
+          <t>Pair-resolvers cannot be evaluated. This is absence of evidence, not genuine divergence. HIGH cardinality is read per active pair from sheet 2. ④-A is reachable ONLY when all defined HIGH resolvers DIVERGE at PRIMARY × PRIMARY with quality ≥ 0.5, except the one-HIGH pair which is intercepted by DEC-7. No Contradiction record is emitted from this coverage outcome.</t>
         </is>
       </c>
     </row>
@@ -7819,7 +9679,7 @@
       </c>
       <c r="D11" s="34" t="inlineStr">
         <is>
-          <t>v3.1: line-level-tier respondent E pattern on governance/resource axes is the EXPECTED outcome of role-tier observation scope. Not a coverage failure — the structural reality.</t>
+          <t>Line-level × Q1 / Q5 default UseClass is CONTEXTUAL (sheet 11). Systematic line-level E on Q1/Q5 is the expected structural outcome of operational altitude, not by itself a coverage failure, and is not a seniority-as-quality penalty.</t>
         </is>
       </c>
     </row>
@@ -7875,7 +9735,7 @@
       </c>
       <c r="B14" s="34" t="inlineStr">
         <is>
-          <t>Combined evidence-quality multiplier from sheet 4 is &lt; 0.4 on ≥ 8 of 11 questions</t>
+          <t>≥ 8 of 11 questions have PRIMARY × PRIMARY comparable comparison unavailable OR provisional PRIMARY × PRIMARY four-factor score &lt; 0.4. Number 8/11 unchanged. DEC-8 PRIMARY × CONTEXTUAL state-③ check is not counted here.</t>
         </is>
       </c>
       <c r="C14" s="34" t="inlineStr">
@@ -7885,7 +9745,7 @@
       </c>
       <c r="D14" s="34" t="inlineStr">
         <is>
-          <t>v3.1: low-quality evidence on most questions means the divergence pattern is unreliable. Do NOT issue Contradiction records. Engagement requires additional respondents or evidence before this comparator yields useful output.</t>
+          <t>Updated coverage predicate (number 8/11 retained): a question counts as insufficient if PRIMARY × PRIMARY comparison is unavailable OR provisional PRIMARY × PRIMARY score &lt; 0.4. If ≥ 8 of 11: COVERAGE INSUFFICIENT. Do NOT issue Contradiction records. DEC-8 PRIMARY × CONTEXTUAL quality-admissibility checks are excluded from this count.</t>
         </is>
       </c>
     </row>
@@ -7906,7 +9766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="14" min="1" max="1"/>
@@ -8259,7 +10119,7 @@
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>ALL multipliers (v3.1 NEW); dimension 5 points to 11_Role_Question_Scope</t>
+          <t>Dim1–dim4 multipliers retained; dim5 SUPERSEDED (DEC-1); four-factor product PROVISIONAL</t>
         </is>
       </c>
       <c r="C16" s="26" t="inlineStr">
@@ -8269,7 +10129,7 @@
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>Direct-observation share, triangulation, confidence, reliability flags, role coverage. Role-coverage dimension 5 source is 11_Role_Question_Scope. Matrix row content status: PENDING SEPARATE AUTHORING ACT. No default/fallback/1.0 substitution for a missing roleCoverageMultiplier.</t>
+          <t>Direct-observation, knowledge-level, confidence, reliability flags remain multiplicative. Role-coverage dimension SUPERSEDED BY OBSERVATION SCOPE LAYER — DEC-1. No roleCoverageMultiplier. Supersedes, does not retract, historical dim-5 text.</t>
         </is>
       </c>
       <c r="E16" s="26" t="inlineStr">
@@ -8475,7 +10335,7 @@
       </c>
       <c r="B24" s="32" t="inlineStr">
         <is>
-          <t>Seniority Tier Mapping + Role_Question_Observation_Scope header-only matrix</t>
+          <t>Superseded D0_R0 matrix-structure placeholder; replaced by D0_R1 rules layer (see r26)</t>
         </is>
       </c>
       <c r="C24" s="32" t="inlineStr">
@@ -8485,12 +10345,12 @@
       </c>
       <c r="D24" s="32" t="inlineStr">
         <is>
-          <t>MATRIX STRUCTURE ONLY — SEPARATE AUTHORING REQUIRED. Zero matrix data rows in this act.</t>
+          <t>Historical D0_R0 row. Current controlling sheet 11 content is the D0_R1 rules layer.</t>
         </is>
       </c>
       <c r="E24" s="32" t="inlineStr">
         <is>
-          <t>NEW — D0_R0</t>
+          <t>SUPERSEDED — D0_R1</t>
         </is>
       </c>
     </row>
@@ -8518,6 +10378,87 @@
       <c r="E25" s="32" t="inlineStr">
         <is>
           <t>NEW — D0_R0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>11_Role_Question_Scope</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Observation Scope rules layer Blocks A/B/C1/C2/C3; seniority mapping retained; roleCoverageMultiplier removed</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>Owner-accepted Dual evidence architecture D0_R1 (DEC-1…DEC-8, DEC-7b, X-9)</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr">
+        <is>
+          <t>MATERIALIZED METHODOLOGY / GENERATED CORPUS. NOT PRODUCTION-ACTIVE — X-3 S-1/S-2 remain open. Supersedes, does not retract, prior role-coverage multiplier language.</t>
+        </is>
+      </c>
+      <c r="E26" s="32" t="inlineStr">
+        <is>
+          <t>CORRECTED — D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>4_Evidence_Quality_Layer</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>Role-coverage dimension SUPERSEDED; provisional four-factor product; 0.027 range ANNULLED; DEC-8 gate documented</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>DEC-1; DEC-8; C-25/X-4 remains OPEN</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="inlineStr">
+        <is>
+          <t>Thresholds 0.7 / 0.5 / 0.4 / 0.2 retained. No replacement range. Four-factor product remains PROVISIONAL.</t>
+        </is>
+      </c>
+      <c r="E27" s="32" t="inlineStr">
+        <is>
+          <t>CORRECTED — D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>12_Classification_Precedence</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>Inserted 0c (UNRESOLVED) and 3a (one-HIGH Q11 DEC-7) with first-match termination</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>DEC-7; DEC-4; X-9</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>Five-state enum unchanged. 3a is routing_outcome, not a new divergence state.</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>CORRECTED — D0_R1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete C5 production interpretation composition
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Dual_Respondent_Axis_Comparison_v1.xlsx
+++ b/NewLogic 03.05.2026/ST_Dual_Respondent_Axis_Comparison_v1.xlsx
@@ -760,12 +760,12 @@
       </c>
       <c r="B12" s="32" t="inlineStr">
         <is>
-          <t>Per-answer environment-signal lookup for all 11 v3.1 AEM/TSAM questions.</t>
+          <t>Per-answer environment-signal lookup for Q1–Q8 and Q11. Q9/Q10 are module-local questionnaire references, not a generic Dual AEM/TSAM map.</t>
         </is>
       </c>
       <c r="C12" s="32" t="inlineStr">
         <is>
-          <t>ST_Acquirer_Environment_Module.xlsx → 3_Screening (signal column)</t>
+          <t>AEM/TSAM 3_Screening for Dual Q1–Q8/Q11 lookup. Q9/Q10 semantic authority remains in the module questionnaires (AEM v3.1 / TSAM).</t>
         </is>
       </c>
       <c r="D12" s="32" t="inlineStr">
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="14" min="1" max="1"/>
@@ -1454,6 +1454,28 @@
       <c r="D21" s="34" t="inlineStr">
         <is>
           <t>Do not close X-2 in this workbook. Canonical Schema unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Q9/Q10 module-aware Dual semantic repair (C5-B.2B + CORR1 + CORR2)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BOUNDED REPAIR — Dual generic Q9/Q10 map removed from active authority</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Four module-local bindings. CORR1 PRE_DUAL_SEMANTIC_INTEGRITY. CORR2 binding digest contract. Both modules Q9-B = STJ/STP·SFP/SFJ. Historical Dual Q9-B NT/STJ secondary origin UNKNOWN. Q1–Q8/Q11 Dual lookup, pair tiers, precedence, Q11, and P_1B unchanged.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Independent verification required. No C5-C, selector, C4, Q11, P_1B, observation-scope, or assembler semantic ownership change.</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="14" min="1" max="1"/>
@@ -1846,6 +1868,28 @@
       <c r="D19" s="32" t="inlineStr">
         <is>
           <t>DEC-1…DEC-8, DEC-7b, X-9, question-qualified E/F, Observation Scope rules layer. Supersedes, does not retract, prior role-coverage multiplier language. 0.027 range SUPERSEDED / ANNULLED — no replacement pending C-25/X-4. Four-factor product remains PROVISIONAL. C-25/X-4 OPEN. X-3 OPEN (S-1/S-2 block production-active Observation Scope). X-8 calibration/schema work remains pending. X-9b UI debt remains open (ST_Step3_Output_Screens_Spec.xlsx / reporting.json not edited). X-10 closure; X-11 closure (Owner-accepted). X-1 / X-2 / X-2b / X-3 not repaired. No empirical validation claimed. No runtime implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>16. C5-B.2B + CORR1 + CORR2 Dual Q9/Q10 module-aware semantic repair</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>REPAIRED</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>sheets 0, 1, 2, 3, 8, 9, 10</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Generic Dual Q9/Q10 answer map removed from active authority and replaced with four module-local questionnaire bindings. Letter AGREE/DIVERGE preserved. Pair/question/HIGH-STANDARD tiers preserved. Classification precedence unchanged. Q9-E/F and Q10-E locks unchanged. CORR1: malformed semantic identity fails PRE_DUAL as INPUT_ASSEMBLY_FAILURE and is not 0c. CORR2: binding digest hashes questionnaire-owned fields plus Dual-owned semanticClass with absent A–D as null. Historical origin of superseded generic/hybrid rows: UNKNOWN.</t>
         </is>
       </c>
     </row>
@@ -4364,14 +4408,14 @@
     <row r="1" ht="31.5" customHeight="1" s="15">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>ANSWER → ENVIRONMENT MAP · v3.1 AEM/TSAM 11 questions · 50+ option cells</t>
+          <t>ANSWER → ENVIRONMENT MAP · v3.1 Dual Q1–Q8/Q11 lookup + Q9/Q10 module-local references</t>
         </is>
       </c>
     </row>
     <row r="2" ht="78" customHeight="1" s="15">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Direct extract from ST_Acquirer_Environment_Module.xlsx → 3_Screening, signal column. v3.1 changes vs source v1.0: all 9 occurrences of "SFP_SFJ" (underscore) corrected to "SFP/SFJ" (slash) per canonical schema; Q11 added (was absent in source v1.0); Option E/F rows added with no_environment_signal mapping; canonical environment names appended in column 7.</t>
+          <t>Q1–Q8 and Q11 remain Dual lookup rows. Q9/Q10 generic Dual answer semantics are removed from active authority. Q9/Q10 resolve only through four module-local questionnaire bindings (AEM Q9, AEM Q10, TSAM Q9, TSAM Q10). Dual does not own a second generic Q9/Q10 answer-semantic truth. Historical origin of the superseded generic/hybrid Q9/Q10 rows: UNKNOWN. Dual Q9-B secondary NT/STJ had no verified source and is not labelled a typo.</t>
         </is>
       </c>
     </row>
@@ -6184,464 +6228,304 @@
     <row r="47" ht="15" customHeight="1" s="15">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>moduleId</t>
         </is>
       </c>
       <c r="B47" s="32" t="inlineStr">
         <is>
-          <t>Confirmatory — STJ/STP vs NT/STJ</t>
+          <t>canonicalQuestionId</t>
         </is>
       </c>
       <c r="C47" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>workbookQuestionId</t>
         </is>
       </c>
       <c r="D47" s="32" t="inlineStr">
         <is>
-          <t>Found better environment — departure as loss</t>
+          <t>sourceWorkbook</t>
         </is>
       </c>
       <c r="E47" s="32" t="inlineStr">
         <is>
-          <t>NT/STJ</t>
+          <t>sourceSheet</t>
         </is>
       </c>
       <c r="F47" s="32" t="inlineStr">
         <is>
-          <t>NF/NT</t>
+          <t>sourceRows</t>
         </is>
       </c>
       <c r="G47" s="32" t="inlineStr">
         <is>
-          <t>The Performance Arena · The Idea Lab</t>
+          <t>sourceVersion</t>
         </is>
       </c>
       <c r="H47" s="32" t="inlineStr">
         <is>
-          <t>SHARED</t>
+          <t>mappingOwner</t>
         </is>
       </c>
     </row>
     <row r="48" ht="23.85" customHeight="1" s="15">
       <c r="A48" s="25" t="inlineStr">
         <is>
+          <t>acquirerEnvironment</t>
+        </is>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>ACQUIRERENVIRONMENT-Q9</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
           <t>Q9</t>
         </is>
       </c>
-      <c r="B48" s="26" t="inlineStr">
-        <is>
-          <t>Confirmatory — STJ/STP vs NT/STJ</t>
-        </is>
-      </c>
-      <c r="C48" s="26" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="D48" s="26" t="inlineStr">
         <is>
-          <t>Became visible as not rising — natural selection</t>
+          <t>ST_Acquirer_Environment_Module.xlsx</t>
         </is>
       </c>
       <c r="E48" s="26" t="inlineStr">
         <is>
-          <t>STJ/STP</t>
+          <t>3_Screening</t>
         </is>
       </c>
       <c r="F48" s="26" t="inlineStr">
         <is>
-          <t>NT/STJ</t>
+          <t>161-166</t>
         </is>
       </c>
       <c r="G48" s="26" t="inlineStr">
         <is>
-          <t>The Power Racket · The Performance Arena (competitive variant)</t>
+          <t>v3.1</t>
         </is>
       </c>
       <c r="H48" s="26" t="inlineStr">
         <is>
-          <t>SHARED — CRITICAL · most important post-close treatment predictor</t>
+          <t>QUESTIONNAIRE_MODULE</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="15">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>acquirerEnvironment</t>
         </is>
       </c>
       <c r="B49" s="32" t="inlineStr">
         <is>
-          <t>Confirmatory — STJ/STP vs NT/STJ</t>
+          <t>ACQUIRERENVIRONMENT-Q10</t>
         </is>
       </c>
       <c r="C49" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="D49" s="32" t="inlineStr">
         <is>
-          <t>Pace and approval requirements incompatible</t>
+          <t>ST_Acquirer_Environment_Module.xlsx</t>
         </is>
       </c>
       <c r="E49" s="32" t="inlineStr">
         <is>
-          <t>NT/STP</t>
+          <t>3_Screening</t>
         </is>
       </c>
       <c r="F49" s="32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>181-185</t>
         </is>
       </c>
       <c r="G49" s="32" t="inlineStr">
         <is>
-          <t>The Disruption Lab</t>
+          <t>v3.1</t>
         </is>
       </c>
       <c r="H49" s="32" t="inlineStr">
         <is>
-          <t>SINGLE</t>
+          <t>QUESTIONNAIRE_MODULE</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="15">
       <c r="A50" s="25" t="inlineStr">
         <is>
+          <t>targetSelfAssessment</t>
+        </is>
+      </c>
+      <c r="B50" s="26" t="inlineStr">
+        <is>
+          <t>TARGETSELFASSESSMENT-Q9</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
           <t>Q9</t>
         </is>
       </c>
-      <c r="B50" s="26" t="inlineStr">
-        <is>
-          <t>Confirmatory — STJ/STP vs NT/STJ</t>
-        </is>
-      </c>
-      <c r="C50" s="26" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="D50" s="26" t="inlineStr">
         <is>
-          <t>Relationship rupture</t>
+          <t>ST_Target_Self_Assessment_Module.xlsx</t>
         </is>
       </c>
       <c r="E50" s="26" t="inlineStr">
         <is>
-          <t>SFJ/SFP</t>
+          <t>3_Screening</t>
         </is>
       </c>
       <c r="F50" s="26" t="inlineStr">
         <is>
-          <t>NF/SFJ</t>
+          <t>161-166</t>
         </is>
       </c>
       <c r="G50" s="26" t="inlineStr">
         <is>
-          <t>The Hometown Network · The Mission Field</t>
+          <t>v3.1</t>
         </is>
       </c>
       <c r="H50" s="26" t="inlineStr">
         <is>
-          <t>SHARED</t>
+          <t>QUESTIONNAIRE_MODULE</t>
         </is>
       </c>
     </row>
     <row r="51" ht="23.85" customHeight="1" s="15">
       <c r="A51" s="33" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>targetSelfAssessment</t>
         </is>
       </c>
       <c r="B51" s="34" t="inlineStr">
         <is>
-          <t>Confirmatory — STJ/STP vs NT/STJ</t>
+          <t>TARGETSELFASSESSMENT-Q10</t>
         </is>
       </c>
       <c r="C51" s="34" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="D51" s="34" t="inlineStr">
         <is>
-          <t>No such departure in observation</t>
+          <t>ST_Target_Self_Assessment_Module.xlsx</t>
         </is>
       </c>
       <c r="E51" s="34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3_Screening</t>
         </is>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>181-185</t>
         </is>
       </c>
       <c r="G51" s="34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>v3.1</t>
         </is>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
-          <t>EXCLUDED — flagged no_such_event_observed</t>
+          <t>QUESTIONNAIRE_MODULE</t>
         </is>
       </c>
     </row>
     <row r="52" ht="23.85" customHeight="1" s="15">
       <c r="A52" s="33" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>HISTORICAL_ORIGIN</t>
         </is>
       </c>
       <c r="B52" s="34" t="inlineStr">
         <is>
-          <t>Confirmatory — STJ/STP vs NT/STJ</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="C52" s="34" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D52" s="34" t="inlineStr">
         <is>
-          <t>Departure occurred but mechanism unknown</t>
+          <t>superseded generic Dual Q9/Q10 map</t>
         </is>
       </c>
       <c r="E52" s="34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>not authoritative</t>
         </is>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="G52" s="34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
-          <t>EXCLUDED — flagged mechanism_unknown</t>
+          <t>Q9-B Dual secondary NT/STJ had no verified source; not labelled a typo.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="15">
-      <c r="A53" s="31" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B53" s="32" t="inlineStr">
-        <is>
-          <t>Confirmatory — NF/SFJ vs NF/NT</t>
-        </is>
-      </c>
-      <c r="C53" s="32" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D53" s="32" t="inlineStr">
-        <is>
-          <t>Work evaluated on merits — thesis revised</t>
-        </is>
-      </c>
-      <c r="E53" s="32" t="inlineStr">
-        <is>
-          <t>NF/NT</t>
-        </is>
-      </c>
-      <c r="F53" s="32" t="inlineStr">
-        <is>
-          <t>NT/STJ</t>
-        </is>
-      </c>
-      <c r="G53" s="32" t="inlineStr">
-        <is>
-          <t>The Idea Lab · The Performance Arena</t>
-        </is>
-      </c>
-      <c r="H53" s="32" t="inlineStr">
-        <is>
-          <t>SHARED — PRIMARY DISCRIMINATOR</t>
-        </is>
-      </c>
+      <c r="A53" s="31" t="n"/>
+      <c r="B53" s="32" t="n"/>
+      <c r="C53" s="32" t="n"/>
+      <c r="D53" s="32" t="n"/>
+      <c r="E53" s="32" t="n"/>
+      <c r="F53" s="32" t="n"/>
+      <c r="G53" s="32" t="n"/>
+      <c r="H53" s="32" t="n"/>
     </row>
     <row r="54" ht="23.85" customHeight="1" s="15">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>Confirmatory — NF/SFJ vs NF/NT</t>
-        </is>
-      </c>
-      <c r="C54" s="26" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D54" s="26" t="inlineStr">
-        <is>
-          <t>Work taken seriously but thesis not challenged</t>
-        </is>
-      </c>
-      <c r="E54" s="26" t="inlineStr">
-        <is>
-          <t>NT/STJ</t>
-        </is>
-      </c>
-      <c r="F54" s="26" t="inlineStr">
-        <is>
-          <t>SFJ/SFP</t>
-        </is>
-      </c>
-      <c r="G54" s="26" t="inlineStr">
-        <is>
-          <t>The Performance Arena · The Hometown Network</t>
-        </is>
-      </c>
-      <c r="H54" s="26" t="inlineStr">
-        <is>
-          <t>SHARED</t>
-        </is>
-      </c>
+      <c r="A54" s="25" t="n"/>
+      <c r="B54" s="26" t="n"/>
+      <c r="C54" s="26" t="n"/>
+      <c r="D54" s="26" t="n"/>
+      <c r="E54" s="26" t="n"/>
+      <c r="F54" s="26" t="n"/>
+      <c r="G54" s="26" t="n"/>
+      <c r="H54" s="26" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="15">
-      <c r="A55" s="31" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B55" s="32" t="inlineStr">
-        <is>
-          <t>Confirmatory — NF/SFJ vs NF/NT</t>
-        </is>
-      </c>
-      <c r="C55" s="32" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D55" s="32" t="inlineStr">
-        <is>
-          <t>Analyst repositioned as not understanding</t>
-        </is>
-      </c>
-      <c r="E55" s="32" t="inlineStr">
-        <is>
-          <t>NF/SFJ</t>
-        </is>
-      </c>
-      <c r="F55" s="32" t="inlineStr">
-        <is>
-          <t>STP/STJ</t>
-        </is>
-      </c>
-      <c r="G55" s="32" t="inlineStr">
-        <is>
-          <t>The Mission Field · The Enforcer Network</t>
-        </is>
-      </c>
-      <c r="H55" s="32" t="inlineStr">
-        <is>
-          <t>SHARED — HIGH RISK</t>
-        </is>
-      </c>
+      <c r="A55" s="31" t="n"/>
+      <c r="B55" s="32" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="32" t="n"/>
+      <c r="H55" s="32" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="15">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B56" s="26" t="inlineStr">
-        <is>
-          <t>Confirmatory — NF/SFJ vs NF/NT</t>
-        </is>
-      </c>
-      <c r="C56" s="26" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D56" s="26" t="inlineStr">
-        <is>
-          <t>Thesis reflects values — analysis informs execution</t>
-        </is>
-      </c>
-      <c r="E56" s="26" t="inlineStr">
-        <is>
-          <t>NF/SFJ</t>
-        </is>
-      </c>
-      <c r="F56" s="26" t="inlineStr">
-        <is>
-          <t>STJ/STP</t>
-        </is>
-      </c>
-      <c r="G56" s="26" t="inlineStr">
-        <is>
-          <t>The Mission Field · The Power Racket</t>
-        </is>
-      </c>
-      <c r="H56" s="26" t="inlineStr">
-        <is>
-          <t>SHARED — HIGH RISK</t>
-        </is>
-      </c>
+      <c r="A56" s="25" t="n"/>
+      <c r="B56" s="26" t="n"/>
+      <c r="C56" s="26" t="n"/>
+      <c r="D56" s="26" t="n"/>
+      <c r="E56" s="26" t="n"/>
+      <c r="F56" s="26" t="n"/>
+      <c r="G56" s="26" t="n"/>
+      <c r="H56" s="26" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="15">
-      <c r="A57" s="33" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B57" s="34" t="inlineStr">
-        <is>
-          <t>Confirmatory — NF/SFJ vs NF/NT</t>
-        </is>
-      </c>
-      <c r="C57" s="34" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D57" s="34" t="inlineStr">
-        <is>
-          <t>Cannot answer from direct observation</t>
-        </is>
-      </c>
-      <c r="E57" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G57" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="34" t="inlineStr">
-        <is>
-          <t>EXCLUDED</t>
-        </is>
-      </c>
+      <c r="A57" s="33" t="n"/>
+      <c r="B57" s="34" t="n"/>
+      <c r="C57" s="34" t="n"/>
+      <c r="D57" s="34" t="n"/>
+      <c r="E57" s="34" t="n"/>
+      <c r="F57" s="34" t="n"/>
+      <c r="G57" s="34" t="n"/>
+      <c r="H57" s="34" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="15">
       <c r="A58" s="25" t="inlineStr">
@@ -7150,12 +7034,12 @@
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>A → NT/STJ</t>
+          <t>Module-local (not generic Dual): AEM Q9-A = STP/STJ·NT/STJ; TSAM Q9-A = NT/STJ·NF/NT</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>C → NT/STP</t>
+          <t>Module-local: AEM Q9-C = STJ/STP (not NT/STP); TSAM Q9-C = NT/STP</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
@@ -7175,7 +7059,7 @@
       </c>
       <c r="I8" s="26" t="inlineStr">
         <is>
-          <t>Q9-C single NT/STP</t>
+          <t>STANDARD tier unchanged. Direction is module-local questionnaire semantics, not generic Dual Q9. Q9-C is NT/STP only in TSAM.</t>
         </is>
       </c>
     </row>
@@ -7432,12 +7316,12 @@
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>A → NT/STJ</t>
+          <t>Module-local: both modules Q9-A include NT/STJ (AEM primary STP/STJ; TSAM primary NT/STJ)</t>
         </is>
       </c>
       <c r="E14" s="26" t="inlineStr">
         <is>
-          <t>B → STJ/STP</t>
+          <t>Module-local: both modules Q9-B = STJ/STP·SFP/SFJ (not Dual hybrid NT/STJ)</t>
         </is>
       </c>
       <c r="F14" s="26" t="inlineStr">
@@ -7457,7 +7341,7 @@
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
-          <t>Most important post-close leadership treatment predictor</t>
+          <t>HIGH — PRIMARY unchanged. A/B identify pair direction in both modules; secondary signals are module-local. Historical Dual Q9-B NT/STJ secondary: UNKNOWN origin.</t>
         </is>
       </c>
     </row>
@@ -7573,12 +7457,12 @@
       </c>
       <c r="D17" s="32" t="inlineStr">
         <is>
-          <t>A → NF/NT·NT/STJ</t>
+          <t>Module-local: both modules Q10-A = NF/NT·NT/STJ</t>
         </is>
       </c>
       <c r="E17" s="32" t="inlineStr">
         <is>
-          <t>C or D → NF/SFJ</t>
+          <t>Module-local: AEM Q10 NF/SFJ is D only; TSAM Q10 NF/SFJ is C and D</t>
         </is>
       </c>
       <c r="F17" s="32" t="inlineStr">
@@ -7598,7 +7482,7 @@
       </c>
       <c r="I17" s="32" t="inlineStr">
         <is>
-          <t>AEM Q10 note: most cognitively demanding; primary discriminator</t>
+          <t>HIGH — PRIMARY unchanged. Generic Dual C/D→NF/SFJ is not AEM-true. Cited AEM Q10 cognitive-demand note is not present in current AEM; that wording is TSAM.</t>
         </is>
       </c>
     </row>
@@ -7813,7 +7697,7 @@
       </c>
       <c r="E22" s="32" t="inlineStr">
         <is>
-          <t>C or D → NF/SFJ</t>
+          <t>Module-local: AEM Q10 only D contains NF/SFJ; TSAM C/D contain NF/SFJ; Q10 has no NF/SFP signal</t>
         </is>
       </c>
       <c r="F22" s="32" t="inlineStr">
@@ -7833,7 +7717,7 @@
       </c>
       <c r="I22" s="32" t="inlineStr">
         <is>
-          <t>Q10 has no NF/SFP signal — Q11 is the only test</t>
+          <t>STANDARD unchanged. Q11 remains the sole HIGH discriminator. Q10 is not a Q11 proxy.</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8181,7 @@
       </c>
       <c r="H13" s="32" t="inlineStr">
         <is>
-          <t>{A,B} split across the two respondents (unordered) is the definitive NT/STJ vs STJ/STP diverge — most important post-close leadership treatment predictor. Both-E in this pair is itself a STJ/STP indicator (departures structurally suppressed).</t>
+          <t>{A,B} letter split remains Dual AGREE/DIVERGE. Environment direction is module-local: both modules Q9-B = STJ/STP·SFP/SFJ; AEM Q9-A = STP/STJ·NT/STJ; TSAM Q9-A = NT/STJ·NF/NT. Generic Dual Q9 map is not authority. Q9-E = EVENT_ABSENCE and Q9-F = OBSERVATION_GAP remain distinct and signal-free.</t>
         </is>
       </c>
     </row>
@@ -8339,7 +8223,7 @@
       </c>
       <c r="H14" s="26" t="inlineStr">
         <is>
-          <t>{A} vs {C/D} split across the two respondents (unordered) is the definitive NF/NT vs NF/SFJ diverge. C and D indicate ideological orthodoxy.</t>
+          <t>{A} vs {C/D} letter split remains Dual AGREE/DIVERGE. Environment direction is module-local: AEM Q10-C = STJ/STP·SFP/SFJ; AEM Q10-D = STP/STJ·NF/SFJ; TSAM Q10-C/D contain NF/SFJ. Generic Dual Q10 map is not authority. Q10-E remains AMBIGUOUS_COLLAPSE and signal-free.</t>
         </is>
       </c>
     </row>
@@ -9766,7 +9650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="14" min="1" max="1"/>
@@ -9822,7 +9706,7 @@
       </c>
       <c r="B5" s="32" t="inlineStr">
         <is>
-          <t>All option-to-environment mappings, Q1-Q10</t>
+          <t>Option-to-environment mappings, Q1–Q8 and Q11</t>
         </is>
       </c>
       <c r="C5" s="32" t="inlineStr">
@@ -9837,7 +9721,7 @@
       </c>
       <c r="E5" s="32" t="inlineStr">
         <is>
-          <t>DIRECT EXTRACT — no interpretation</t>
+          <t>DIRECT EXTRACT for Dual Q1–Q8/Q11 lookup rows from cited AEM 3_Screening where still accurate. Q9/Q10 generic Dual map is not a direct AEM extract and is not active authority.</t>
         </is>
       </c>
     </row>
@@ -9962,17 +9846,17 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>ST_Acquirer_Environment_Module.xlsx</t>
+          <t>ST_Acquirer_Environment_Module.xlsx (Q2); Q9 semantic authority is module-local AEM/TSAM questionnaires</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>Q2 ℹ note: "single most reliable acquirer environment discriminator"; Q9 ℹ note: "most important post-close treatment predictor"</t>
+          <t>Q2 ℹ note remains the Dual HIGH-tier source. Cited AEM Q9 'post-close treatment' note is not present in current AEM. Q9 HIGH tier is preserved; Q9 answer semantics are module-local.</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
         <is>
-          <t>DIRECT EXTRACT</t>
+          <t>DIRECT EXTRACT for Q2 HIGH tier; Q9 semantics = MODULE_LOCAL_REFERENCE</t>
         </is>
       </c>
     </row>
@@ -10016,17 +9900,17 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>ST_Acquirer_Environment_Module.xlsx</t>
+          <t>Q10 HIGH tier is Dual pair-weight authority; Q10 answer semantics are module-local AEM/TSAM questionnaires</t>
         </is>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>Q10 cognitive-demand note + Q8-D single NF/SFJ signal</t>
+          <t>Q10 HIGH tier preserved. Cited AEM Q10 cognitive-demand note is not present in current AEM; that wording is TSAM. AEM Q10-C is not NF/SFJ.</t>
         </is>
       </c>
       <c r="E12" s="26" t="inlineStr">
         <is>
-          <t>DIRECT EXTRACT</t>
+          <t>DIRECT EXTRACT for Q8-D NF/SFJ signal; Q10 semantics = MODULE_LOCAL_REFERENCE</t>
         </is>
       </c>
     </row>
@@ -10459,6 +10343,141 @@
       <c r="E28" s="32" t="inlineStr">
         <is>
           <t>CORRECTED — D0_R1</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1_Answer_Env_Map</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AEM Q9 module-local binding ACQUIRERENVIRONMENT-Q9</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ST_Acquirer_Environment_Module.xlsx</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>3_Screening rows 161-166; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1_Answer_Env_Map</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AEM Q10 module-local binding ACQUIRERENVIRONMENT-Q10</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ST_Acquirer_Environment_Module.xlsx</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>3_Screening rows 181-185; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1_Answer_Env_Map</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TSAM Q9 module-local binding TARGETSELFASSESSMENT-Q9</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ST_Target_Self_Assessment_Module.xlsx</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>3_Screening rows 161-166; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1_Answer_Env_Map</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TSAM Q10 module-local binding TARGETSELFASSESSMENT-Q10</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ST_Target_Self_Assessment_Module.xlsx</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>3_Screening rows 181-185; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1_Answer_Env_Map</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Superseded generic Dual Q9/Q10 rows, including Dual Q9-B secondary NT/STJ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No verified AEM or TSAM source for the generic Dual Q9/Q10 map or the Q9-B NT/STJ secondary</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SUPERSEDED — historical origin UNKNOWN; not labelled a typo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: implement canonical homogeneous semantics
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Dual_Respondent_Axis_Comparison_v1.xlsx
+++ b/NewLogic 03.05.2026/ST_Dual_Respondent_Axis_Comparison_v1.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_v3_1_Build_Notes" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Role_Question_Scope" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Classification_Precedence" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Cross_Side_Structural_Diff" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1458,22 +1459,22 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Q9/Q10 module-aware Dual semantic repair (C5-B.2B + CORR1 + CORR2)</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>BOUNDED REPAIR — Dual generic Q9/Q10 map removed from active authority</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Four module-local bindings. CORR1 PRE_DUAL_SEMANTIC_INTEGRITY. CORR2 binding digest contract. Both modules Q9-B = STJ/STP·SFP/SFJ. Historical Dual Q9-B NT/STJ secondary origin UNKNOWN. Q1–Q8/Q11 Dual lookup, pair tiers, precedence, Q11, and P_1B unchanged.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Independent verification required. No C5-C, selector, C4, Q11, P_1B, observation-scope, or assembler semantic ownership change.</t>
         </is>
@@ -1872,22 +1873,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>16. C5-B.2B + CORR1 + CORR2 Dual Q9/Q10 module-aware semantic repair</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>REPAIRED</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>sheets 0, 1, 2, 3, 8, 9, 10</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Generic Dual Q9/Q10 answer map removed from active authority and replaced with four module-local questionnaire bindings. Letter AGREE/DIVERGE preserved. Pair/question/HIGH-STANDARD tiers preserved. Classification precedence unchanged. Q9-E/F and Q10-E locks unchanged. CORR1: malformed semantic identity fails PRE_DUAL as INPUT_ASSEMBLY_FAILURE and is not 0c. CORR2: binding digest hashes questionnaire-owned fields plus Dual-owned semanticClass with absent A–D as null. Historical origin of superseded generic/hybrid rows: UNKNOWN.</t>
         </is>
@@ -4387,6 +4388,208 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CROSS-SIDE STRUCTURAL DIFFERENTIATION · AEM ↔ TSAM · Cross_Side_Structural_Differentiation v1</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GOVERNED SHEET added under Owner decisions OD-RMP3-1…OD-RMP3-16 (RMP-3 core implementation, accepted August 2026). Amendment adds this sheet only; no existing sheet of this workbook changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Governed rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>For a same-environment (homogeneous) pair, count the comparable structural answer dimensions on which the Acquirer Environment Module (AEM) and the Target Self-Assessment Module (TSAM) selected different canonical options. Same environment code does not mean same answer pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cross_side: AEM (ST_Acquirer_Environment_Module.xlsx · 3_Screening) ↔ TSAM (ST_Target_Self_Assessment_Module.xlsx · 3_Screening) on the shared question set Q1–Q11, matched by workbookQuestionId. TOD, EDv2, and the canonical 80/20 environment vector are NOT valid bases for this layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Comparison rule</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Letter-level canonical option identity per selected option letter, following sheet 3_Comparison_Engine letter logic: identical letters = AGREE (aligned); different letters = DIVERGE. Q9/Q10 compare the canonical selected letter only; their module-local environment mappings are not authority cross-side (sheet 1_Answer_Env_Map note and answerSemanticBindings). Cross-side environment-vector distance (L1/L2/cosine/JSD or any full-vector divergence) is forbidden for this layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Comparable options</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Options A–D are comparable. Option E/F comparability is governed by sheet 11_Role_Question_Scope Block C1/C2 semantic classes: comparable when the class preserves ordinary comparison / divergence-map semantics (EXTERNAL_OR_PERSONAL_CAUSE — Q6-E; SUBSTANTIVE_SIGNAL — Q11-E); not comparable when the class states comparable answer unavailable (OBSERVATION_GAP, EVENT_ABSENCE, STRUCTURAL_PRECONDITION_ABSENCE, AMBIGUOUS_COLLAPSE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Row status values</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>aligned = identical comparable letters on both sides. divergent = different comparable letters on both sides. not_comparable = question unanswered/missing on either side, or either selected option is a non-comparable E/F class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Count definitions</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>comparableCount = number of aligned rows + number of divergent rows. agreeCount = number of aligned rows. divergeCount = number of divergent rows. Required arithmetic: agreeCount + divergeCount = comparableCount. Integer counts only; no floats, no 0–100 conversion, no averaging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Missing-data denominator rule</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>not_comparable rows are excluded from the denominator. No substitution, no imputation, no weighting of missing answers. A question answered on one side only is not_comparable, not divergent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Symmetry</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AEM ↔ TSAM order swap preserves comparableCount, agreeCount, and divergeCount exactly. The layer is history independent: only current selected letters matter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>No weights</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>This layer introduces no weights, no thresholds, and no numeric severity. The sheet 4_Evidence_Quality_Layer four-factor product is NOT a differentiation magnitude and must not be used as one; evidence quality remains separate metadata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Explicit non-claims</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NOT ECS. NOT FRICTION. NOT SEVERITY. NOT RESOURCE PRESSURE. NOT a resource-conflict score. This layer does not modify ECS, the ECS range, the risk band, ERI resource tiers, or canonical Net Effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Insufficient evidence</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>When comparableCount = 0 or required cross-side AEM/TSAM evidence is unavailable, emit the structured unavailable state INSUFFICIENT_COMPARABLE_CROSS_SIDE_EVIDENCE. Do not manufacture a score or substitute other instruments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Public representation</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>"{divergeCount} of {comparableCount} comparable structural dimensions differ" plus the exact per-dimension rows (questionId, axis label, both selected options, row status).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Provenance</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NewLogic 03.05.2026 corpus · ST_Dual_Respondent_Axis_Comparison_v1.xlsx. Owner decisions OD-RMP3-1…OD-RMP3-16 (accepted August 2026) · RMP-3 core implementation. Source basis: sheet 3_Comparison_Engine (letter logic), sheet 1_Answer_Env_Map (question identities / axis labels / Q9-Q10 module-local note), sheet 11_Role_Question_Scope Blocks C1/C2 (option semantic classes).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -10347,135 +10550,135 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>1_Answer_Env_Map</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>AEM Q9 module-local binding ACQUIRERENVIRONMENT-Q9</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>ST_Acquirer_Environment_Module.xlsx</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>3_Screening rows 161-166; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>1_Answer_Env_Map</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>AEM Q10 module-local binding ACQUIRERENVIRONMENT-Q10</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>ST_Acquirer_Environment_Module.xlsx</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>3_Screening rows 181-185; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>1_Answer_Env_Map</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>TSAM Q9 module-local binding TARGETSELFASSESSMENT-Q9</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr">
         <is>
           <t>ST_Target_Self_Assessment_Module.xlsx</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>3_Screening rows 161-166; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>1_Answer_Env_Map</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>TSAM Q10 module-local binding TARGETSELFASSESSMENT-Q10</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>ST_Target_Self_Assessment_Module.xlsx</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>3_Screening rows 181-185; mappingOwner=QUESTIONNAIRE_MODULE; derivationType=MODULE_LOCAL_REFERENCE</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>MODULE_LOCAL_REFERENCE — Dual does not copy option signals</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>1_Answer_Env_Map</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Superseded generic Dual Q9/Q10 rows, including Dual Q9-B secondary NT/STJ</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>No verified AEM or TSAM source for the generic Dual Q9/Q10 map or the Q9-B NT/STJ secondary</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>SUPERSEDED — historical origin UNKNOWN; not labelled a typo</t>
         </is>

</xml_diff>